<commit_message>
docs: align backend work plan with Java Spring Boot
</commit_message>
<xml_diff>
--- a/docs/backend-team-checklist.xlsx
+++ b/docs/backend-team-checklist.xlsx
@@ -15,8 +15,9 @@
     <sheet name="Quyet_dinh" sheetId="8" r:id="rId8"/>
     <sheet name="Worker_OPS" sheetId="9" r:id="rId9"/>
     <sheet name="QA" sheetId="10" r:id="rId10"/>
-    <sheet name="FE" sheetId="11" r:id="rId11"/>
-    <sheet name="AI" sheetId="12" r:id="rId12"/>
+    <sheet name="Cau_truc_BE" sheetId="11" r:id="rId11"/>
+    <sheet name="FE" sheetId="12" r:id="rId12"/>
+    <sheet name="AI" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -134,7 +135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -264,48 +265,60 @@
     <row r="11" ht="72" customHeight="1">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">File dùng chung</t>
+          <t xml:space="preserve">Java Spring Boot</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">A tích hợp bootstrap/dependency/CI/output SQL trong chính lượt bàn giao cần nó; không có một task tương lai để chờ sửa provider. B/C sửa source SQL đã phân. backend/** là bố cục đề xuất, chưa phải backend đã có.</t>
+          <t xml:space="preserve">Java 21 LTS + Spring Boot + Maven Wrapper + MySQL; Spring JDBC tích hợp SQL/procedure hiện có. BE-A01 tạo project thật. Sheet Cau_truc_BE mô tả stack, cây thư mục và quy ước.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đồng bộ trang</t>
+          <t xml:space="preserve">File dùng chung</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiến độ trên trang chỉ lưu trong trình duyệt này; Excel không tự đồng bộ với trang hoặc máy khác. Team nên dùng một bản workbook chung hoặc công cụ task làm nguồn thật.</t>
+          <t xml:space="preserve">A tích hợp TrodayApplication/config/shared/pom.xml/Maven Wrapper/application*.yml/CI/output SQL ngay trong lượt bàn giao cần nó. B/C thêm bean trong package chức năng và sửa source SQL đã phân. backend/** là bố cục đề xuất, chưa phải backend đã có.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="72" customHeight="1">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">FE / AI</t>
+          <t xml:space="preserve">Đồng bộ trang</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hai sheet cuối hoàn toàn trống, dành cho lập kế hoạch sau. Không tự phát sinh task FE/AI.</t>
+          <t xml:space="preserve">Tiến độ trên trang chỉ lưu trong trình duyệt này; Excel không tự đồng bộ với trang hoặc máy khác. Team nên dùng một bản workbook chung hoặc công cụ task làm nguồn thật.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="72" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">FE / AI</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hai sheet cuối hoàn toàn trống, dành cho lập kế hoạch sau. Không tự phát sinh task FE/AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">Nguồn</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kế hoạch v2 tuần tự; giữ task ID của v1, đổi STT chung và thứ tự hàng. docs/api-catalog.json + scripts/work-plan-blueprint.cjs → JSON/JS/Excel. Kiểm tra: npm run plan:check; npm run test:work-plan.</t>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kế hoạch v2 tuần tự; giữ thứ tự 52 task khi bổ sung Java Spring Boot. docs/api-catalog.json + scripts/work-plan-blueprint.cjs + scripts/spring-boot-plan.cjs → JSON/JS/Excel. Kiểm tra: npm run plan:check; npm run test:work-plan.</t>
         </is>
       </c>
     </row>
@@ -971,13 +984,1167 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B94"/>
+  <sheetFormatPr defaultRowHeight="20"/>
+  <cols>
+    <col min="1" max="1" width="45" customWidth="1"/>
+    <col min="2" max="2" width="160" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thành phần / quy ước</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Java Spring Boot dự kiến</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Trạng thái</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đã chốt stack cho kế hoạch; repo chưa có ứng dụng Java Spring Boot chạy thật. BE-A01 mới tạo pom.xml, main class và cấu hình.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Version</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BE-A01 chọn bản Spring Boot stable tương thích Java 21 và dependency của dự án, pin version trong pom.xml/Maven Wrapper. Không dùng SNAPSHOT; chưa có pom.xml thực tế để xác nhận patch version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Package gốc</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">com.troday</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ngôn ngữ &amp; build</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Java 21 LTS · Maven Wrapper
+pom.xml, mvnw/mvnw.cmd và .mvn/wrapper do A giữ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP API</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring Web MVC
+@RestController theo chức năng, DTO riêng, envelope chung /api/v1; SSE dùng SseEmitter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validation &amp; lỗi</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jakarta Bean Validation · @RestControllerAdvice
+@Valid trên request DTO; GlobalExceptionHandler trả đúng error code và requestId.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bảo mật</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring Security
+SecurityFilterChain, JWT/session validation và kiểm tra scope đối tượng; actor lấy từ SecurityContext.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Truy cập CSDL</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring JDBC · MySQL Connector/J
+NamedParameterJdbcTemplate cho query/CRUD; SimpleJdbcCall hoặc CallableStatement cho stored procedure hiện có.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giao dịch</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@Transactional / TransactionTemplate + gateway procedure riêng
+Service tự ghi nhiều bảng dùng transaction Spring; CALL tự START/COMMIT chạy ngoài transaction Spring và bị từ chối nếu caller đang có transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiểm thử</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JUnit Jupiter · MockMvc · MySQL test độc lập
+@SpringBootTest cho wiring/integration; Testcontainers MySQL cho CHECK/FK/trigger/procedure, không thay bằng H2 cho ca SQL v5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/                                      # Dự án Spring Boot dự kiến; chưa tạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── pom.xml                                   # A: version, dependency và Maven plugins</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── mvnw / mvnw.cmd / .mvn/wrapper/            # A: cùng một Maven Wrapper cho team</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── docs/contracts/                           # JSON/schema API; mỗi module có file riêng</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── core.json                             # A: envelope/error/type conventions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── identity.json, files.json, messaging.json, notifications.json, billing.json # A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── accountadmin.json, audit.json, admindashboard.json       # A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── properties.json, houserights.json, posts.json, services.json, viewings.json # B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="72" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── roommates.json, reviews.json, reports.json               # B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   └── rentals.json                          # C</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── src/main/java/com/troday/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── TrodayApplication.java                # A: @SpringBootApplication ở package gốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── config/                              # A: Security/DataSource/Scheduling config</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── shared/                              # A: code dùng chung, không chứa nghiệp vụ thuê</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── api/                             # ApiResponse, PageMeta, RequestId</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── error/                           # GlobalExceptionHandler, DomainException</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="72" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── security/                        # ActorContext, scope helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── transaction/                     # StoredProcedureGateway, transaction helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── audit/                           # AuditPort/adapter, target D14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── event/                           # EventPort/outbox adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   ├── idempotency/                     # request key/hash/result store</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   │   └── time/                            # UTC Instant / ngày nghiệp vụ Việt Nam</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── identity/                            # A: tài khoản, phiên, OTP, xác minh</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── files/                               # A: kho tệp, private access, retention</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="72" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── messaging/                           # A: conversation/messages/post share</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── notifications/                       # A: feed, read-state, SSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── billing/                             # A: invoices/invoice_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── accountadmin/ audit/ admindashboard/  # A: user lock, audit query, tổng quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── properties/ houserights/              # B: nhà/phòng, quyền cho thuê</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── posts/ services/ viewings/            # B: tin, giá dịch vụ, lịch xem</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="72" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── roommates/ reviews/ reports/          # B: kết nối/ghép, đánh giá/báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="72" customHeight="1">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   └── rentals/                             # C: mỗi nhóm thuê có package con</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="72" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│       ├── contracts/ revisions/ residents/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="72" customHeight="1">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│       ├── joins/ changes/ representatives/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="72" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│       └── templates/ residencylink/ port/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="72" customHeight="1">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── src/main/resources/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="72" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── application.yml                      # A: cấu hình chung, giá trị qua environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="72" customHeight="1">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   └── application-local.yml                # A: profile local; không commit secret</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="72" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── src/test/java/com/troday/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="72" customHeight="1">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── shared/ config/                      # A: core/config tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="72" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── identity/ files/ messaging/ notifications/ billing/  # A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="72" customHeight="1">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── properties/ services/ posts/ viewings/ roommates/   # B</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── houserights/ reviews/ reports/ sqlproperty/ # B</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── accountadmin/ audit/ admindashboard/   # A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="72" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── sqlrental/                           # C: procedure/trigger tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="72" customHeight="1">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── rentals/                             # C: contract/occupancy/race tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="72" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── support/fixtures/a/ b/ c/             # Fixture Java riêng theo owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="72" customHeight="1">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── contract/a/ b/ c/                     # Contract tests riêng</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="72" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   └── e2e/platform/ property/ viewingcontract/ rental/ release/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="72" customHeight="1">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B61" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── src/test/resources/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="72" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   ├── application-test.yml                 # A: MySQL/kho tệp test độc lập</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="72" customHeight="1">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">│   └── sql/a/ b/ c/                         # SQL fixture theo owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="72" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">└── target/                                  # Maven sinh ra; không commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="72" customHeight="1">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">database/source/*.sql                         # Nguồn SQL hiện có ở root repo: B/C theo owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="72" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cây thư mục BE</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">database/schema.sql + migrations/               # A tích hợp output; không tự sinh schema từ ORM</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="72" customHeight="1">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">com/troday/properties/                        # Ví dụ một module của B</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="72" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── controller/HouseController.java            # @RestController, chỉ HTTP/DTO/scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="72" customHeight="1">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── dto/request/CreateHouseRequest.java        # record + jakarta.validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="72" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── dto/response/HouseResponse.java            # Không trả domain model trực tiếp</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="72" customHeight="1">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── service/HouseService.java                  # @Service, quy tắc và điều phối</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="72" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── repository/HouseRepository.java            # @Repository, SQL/DB mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="72" customHeight="1">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── repository/mapper/HouseRowMapper.java      # RowMapper dùng JDBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="72" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── domain/House.java                          # Model Java thuần, chưa yêu cầu @Entity</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="72" customHeight="1">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">├── port/PropertyReadPort.java                 # Interface công khai cho consumer</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="72" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">└── adapter/PropertyReadJdbcAdapter.java        # Bean đọc riêng, tránh vòng phụ thuộc service</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="72" customHeight="1">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controller → Service → Repository / Procedure adapter → MySQL</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="72" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Một module mẫu</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consumer module → Java Port interface → Adapter của module provider</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="72" customHeight="1">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Main class và package</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt TrodayApplication trong com.troday, các package chức năng nằm bên dưới. Package viết thường, không có dấu gạch nối; dùng houserights/accountadmin thay house-rights/account-admin. Đây là quy ước của team, không phải cấu trúc duy nhất Spring Boot cho phép.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="72" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bean và route theo module</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controller dùng @RestController/@RequestMapping, nghiệp vụ @Service, SQL adapter @Repository; constructor injection. Spring component scan nhận bean dưới package gốc, không có file routes.* hoặc manifest module để ba người cùng sửa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="72" customHeight="1">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DTO, kiểu số và ngày</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request/response DTO riêng, có @Valid và Bean Validation. Tiền dùng BigDecimal; ID trong JSON giữ chuỗi như đặc tả; Instant cho thời điểm UTC, LocalDate cho ngày Việt Nam. Không tự expose model hoặc giấy tờ cá nhân.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="72" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giao dịch do service quản lý</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dùng @Transactional tại service public hoặc TransactionTemplate cho thao tác tự ghi nhiều bảng. Các repository/port dùng cùng DataSource và transaction Spring; không commit riêng trong adapter. Tham số tx trong đặc tả là ngữ cảnh server, không truyền JDBC Connection qua HTTP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="72" customHeight="1">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giao dịch do procedure quản lý</t>
+        </is>
+      </c>
+      <c r="B83" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">StoredProcedureGateway là bean riêng, gọi SimpleJdbcCall/CallableStatement với tham số IN/OUT tường minh. Dùng Propagation.NEVER để fail nếu caller đang có transaction Spring; không bọc CALL tự START/COMMIT trong @Transactional. Test đường gọi qua proxy, không self-invocation bỏ qua guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="72" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tôn trọng SQL hiện có</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MySQL CHECK/FK/trigger và thủ tục là nguồn ràng buộc đã có. Kế hoạch chọn Spring JDBC để tích hợp; không bật Hibernate ddl-auto=create/update hoặc tạo bản entity DDL khác. Nếu bổ sung JPA sau này phải có quyết định riêng về mapping và transaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="72" customHeight="1">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không tạo vòng phụ thuộc bean</t>
+        </is>
+      </c>
+      <c r="B85" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Port đọc được implement bằng adapter/repository riêng; không inject ngược service nghiệp vụ vào nhau và không dùng @Lazy để che vòng phụ thuộc. Test @SpringBootTest phải khởi tạo được application context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="72" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test và cấu hình dùng chung</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JUnit/MockMvc kiểm thử HTTP/security; MySQL test độc lập kiểm thử procedure/race/rollback. A giữ pom.xml, wrapper, main class, config dùng chung và resources profile; B/C giữ package chức năng, test và contract riêng. Lệnh Maven chỉ chạy được sau khi BE-A01 tạo dự án.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="72" customHeight="1">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chạy local sau BE-A01</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd spring-boot:run "-Dspring-boot.run.profiles=local"
+Đã cấu hình MySQL local và biến môi trường.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="72" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unit/controller tests</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd test
+JUnit Jupiter / MockMvc; không dùng DB thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="72" customHeight="1">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiểm thử/bản build tích hợp</t>
+        </is>
+      </c>
+      <c r="B89" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd verify
+BE-A01 cấu hình integration tests và DB MySQL test riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="72" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linux/macOS</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./mvnw test
+Dùng ./mvnw verify khi kiểm thử tích hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="72" customHeight="1">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring Boot: bố trí main class và package</t>
+        </is>
+      </c>
+      <c r="B91" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-boot/reference/using/structuring-your-code.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="72" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring JDBC: SimpleJdbcCall</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/reference/data-access/jdbc/simple.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="72" customHeight="1">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring: Propagation.NEVER</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/docs/current/javadoc-api/org/springframework/transaction/annotation/Propagation.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="72" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring Boot: tương thích Java và build tools</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-boot/system-requirements.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <sheetData/>
@@ -1681,7 +2848,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khởi tạo backend, nhánh và CI theo module</t>
+          <t xml:space="preserve">Khởi tạo Java Spring Boot, Maven và CI</t>
         </is>
       </c>
       <c r="G2" s="2">
@@ -1697,19 +2864,27 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/tests/e2e/release/**</t>
+backend/src/main/resources/application*.yml
+backend/src/test/resources/application-test.yml
+backend/src/test/java/com/troday/e2e/release/**</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1729,15 +2904,15 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tạo backend/src/modules/&lt;domain&gt;, tests/fixtures theo module và manifest tự đăng ký.
-Mỗi PR có branch be/&lt;owner&gt;/&lt;task-id&gt;-&lt;slug&gt;; main được bảo vệ bằng review và CI.
-CI dựng SQL từ nguồn vào thư mục tạm cho feature PR; A giữ output SQL tích hợp khớp nguồn khi merge.</t>
+          <t xml:space="preserve">Tạo backend/pom.xml, Maven Wrapper, TrodayApplication trong com.troday, package chức năng và resources profiles; Spring component scan nhận bean.
+Chọn starters Web MVC/Validation/Security/JDBC, MySQL driver và test tương thích; CI chạy Maven test/verify trên DB test riêng.
+CI dựng SQL nguồn vào thư mục tạm, không bật ORM tự tạo/cập nhật schema; nhánh be/&lt;owner&gt;/&lt;task-id&gt;-&lt;slug&gt; và review bắt buộc.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lệnh chạy và test được ghi trong README backend; không dùng DB thật để test.
-B/C thêm module qua manifest riêng mà không sửa bootstrap, lockfile hay root routes.</t>
+          <t xml:space="preserve">Application context Spring Boot khởi tạo được; mvnw.cmd test/verify và lệnh chạy local được ghi trong README, không dùng DB thật để test.
+B/C thêm controller/service/repository dưới com.troday mà không cùng sửa main class, pom.xml hoặc SecurityConfig.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -1870,26 +3045,29 @@
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*
-backend/src/modules/posts/**
-backend/tests/posts/**
-backend/contracts/posts.*
-backend/src/modules/services/**
-backend/tests/services/**
-backend/contracts/services.*
-backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*
-backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**
+backend/src/main/java/com/troday/posts/**
+backend/src/test/java/com/troday/posts/**
+backend/docs/contracts/posts.json
+backend/src/main/java/com/troday/services/**
+backend/src/test/java/com/troday/services/**
+backend/docs/contracts/services.json
+backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**
+backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K3" s="0" t="inlineStr">
@@ -1910,7 +3088,7 @@
       <c r="N3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Phân biệt postId/roomId, quyền nhà, capacity load, quote service và trạng thái kết nối.
-Tạo fixture trong backend/tests/fixtures/B/**; không sửa seed chung của A/C.
+Tạo fixture trong backend/src/test/java/com/troday/support/fixtures/b/**; không sửa seed chung của A/C.
 Gửi đề xuất IF-ROOM/IF-SERVICE/IF-CONNECTION để C01 phân tích thuê và A02 chốt contract v1 ở các lượt tiếp theo.</t>
         </is>
       </c>
@@ -2050,15 +3228,16 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -2219,15 +3398,21 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
@@ -2247,9 +3432,9 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Công bố backend/contracts/core.* với fixture request/response/error và mock adapter.
-Tách UnitOfWork của service với ProcedureRunner tự START/COMMIT; actor luôn lấy từ phiên.
-Định nghĩa eventId/recipient/eventKey, idempotency scope và whitelist audit target; B/C có contract test dùng ngay.</t>
+          <t xml:space="preserve">Công bố backend/docs/contracts/core.json cùng Java record ActorContext/ApiResponse, DTO validation và error mapping trong shared/.
+Service tự ghi dùng @Transactional/TransactionTemplate; StoredProcedureGateway là bean riêng dùng Propagation.NEVER khi CALL tự START/COMMIT; actor lấy từ SecurityContext.
+Định nghĩa eventId/recipient/eventKey, idempotency scope, whitelist audit target; constructor injection và contract test JUnit sẵn cho B/C.</t>
         </is>
       </c>
       <c r="O5" s="0" t="inlineStr">
@@ -2388,9 +3573,9 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/identity/**
-backend/tests/identity/**
-backend/contracts/identity.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
+backend/src/test/java/com/troday/identity/**
+backend/docs/contracts/identity.json</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2551,19 +3736,27 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/tests/e2e/release/**</t>
+backend/src/main/resources/application*.yml
+backend/src/test/resources/application-test.yml
+backend/src/test/java/com/troday/e2e/release/**</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
@@ -2724,9 +3917,9 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/files/**
-backend/tests/files/**
-backend/contracts/files.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/files/**
+backend/src/test/java/com/troday/files/**
+backend/docs/contracts/files.json</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2887,9 +4080,9 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/identity/**
-backend/tests/identity/**
-backend/contracts/identity.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
+backend/src/test/java/com/troday/identity/**
+backend/docs/contracts/identity.json</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
@@ -3050,9 +4243,9 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/identity/**
-backend/tests/identity/**
-backend/contracts/identity.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
+backend/src/test/java/com/troday/identity/**
+backend/docs/contracts/identity.json</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -3074,7 +4267,7 @@
         <is>
           <t xml:space="preserve">Hash/HMAC mã, hạn dùng, attempt, consumed/revoked; reset không lộ tài khoản tồn tại.
 Reset grant chỉ đổi mật khẩu đúng user và thu hồi phiên; phone uniqueness kiểm tra lại dưới khóa.
-TokenPort issue/consume hỗ trợ OCCUPANT_LINK và targetRoomTenantId trong transaction được C truyền vào.</t>
+TokenPort issue/consume hỗ trợ OCCUPANT_LINK và targetRoomTenantId trong transaction Spring do service C mở, repository A tham gia cùng DataSource.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -3213,13 +4406,16 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**</t>
         </is>
       </c>
       <c r="K11" s="0" t="inlineStr">
@@ -3380,9 +4576,9 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/services/**
-backend/tests/services/**
-backend/contracts/services.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/services/**
+backend/src/test/java/com/troday/services/**
+backend/docs/contracts/services.json</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -3543,19 +4739,22 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*
-backend/src/modules/services/**
-backend/tests/services/**
-backend/contracts/services.*
-backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**
+backend/src/main/java/com/troday/services/**
+backend/src/test/java/com/troday/services/**
+backend/docs/contracts/services.json
+backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
@@ -3716,12 +4915,13 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -3882,12 +5082,13 @@
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
@@ -4048,17 +5249,20 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -4219,13 +5423,13 @@
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/posts/**
-backend/tests/posts/**
-backend/contracts/posts.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
+backend/src/test/java/com/troday/posts/**
+backend/docs/contracts/posts.json
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
@@ -4386,16 +5590,19 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/posts/**
-backend/tests/posts/**
-backend/contracts/posts.*
-backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
+backend/src/test/java/com/troday/posts/**
+backend/docs/contracts/posts.json
+backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -4556,15 +5763,16 @@
       </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K19" s="0" t="inlineStr">
@@ -4585,7 +5793,7 @@
       <c r="N19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Procedure confirm nhận expectedRevisionId và so dưới cùng khóa; stale 409 không xác nhận bản mới.
-Mapper camelCase → SQL params/JSON snake_case; ProcedureRunner không bị bọc UoW ngoài.
+Mapper camelCase → SQL params/JSON snake_case; StoredProcedureGateway là bean riêng có @Transactional(propagation=Propagation.NEVER), không bị bọc transaction Spring ngoài.
 Race/rollback fixture cho create/move-in/handover/transfer; đưa patch source cho A tái sinh SQL trước tích hợp.</t>
         </is>
       </c>
@@ -4725,10 +5933,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -4889,10 +6099,12 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
@@ -5053,14 +6265,14 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -5221,14 +6433,14 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
@@ -5389,15 +6601,16 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -5558,10 +6771,10 @@
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**</t>
         </is>
       </c>
       <c r="K25" s="0" t="inlineStr">
@@ -5722,15 +6935,16 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -5891,15 +7105,16 @@
       </c>
       <c r="J27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K27" s="0" t="inlineStr">
@@ -6060,12 +7275,13 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -6086,7 +7302,7 @@
       <c r="N28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Chủ mời member đúng contract chưa có tenant; OCCUPANT_LINK gắn target room_tenant.
-Tiêu thụ token và gắn account trong UoW của C, gọi A token adapter bằng cùng connection.
+Service C dùng @Transactional/TransactionTemplate để tiêu thụ token và gắn account; token repository A tham gia cùng transaction/DataSource.
 Chốt D06 kênh/đối chiếu người nhận; không gắn tài khoản theo tên tự khai.</t>
         </is>
       </c>
@@ -6226,9 +7442,9 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
@@ -6389,9 +7605,9 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -6552,9 +7768,9 @@
       </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K31" s="0" t="inlineStr">
@@ -6715,10 +7931,12 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -6879,12 +8097,13 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
@@ -7045,9 +8264,9 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/billing/**
-backend/tests/billing/**
-backend/contracts/billing.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
+backend/src/test/java/com/troday/billing/**
+backend/docs/contracts/billing.json</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -7208,10 +8427,15 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/account-admin/**
-backend/src/modules/audit/**
-backend/src/modules/admin-dashboard/**
-backend/tests/account-admin/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/accountadmin/**
+backend/src/test/java/com/troday/accountadmin/**
+backend/src/main/java/com/troday/audit/**
+backend/src/test/java/com/troday/audit/**
+backend/src/main/java/com/troday/admindashboard/**
+backend/src/test/java/com/troday/admindashboard/**
+backend/docs/contracts/accountadmin.json
+backend/docs/contracts/audit.json
+backend/docs/contracts/admindashboard.json</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
@@ -7372,9 +8596,9 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/billing/**
-backend/tests/billing/**
-backend/contracts/billing.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
+backend/src/test/java/com/troday/billing/**
+backend/docs/contracts/billing.json</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -7535,15 +8759,16 @@
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
@@ -7704,15 +8929,16 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -7873,15 +9099,16 @@
       </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K39" s="0" t="inlineStr">
@@ -8042,10 +9269,12 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -8206,9 +9435,12 @@
       </c>
       <c r="J41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/reviews/**
-backend/src/modules/reports/**
-backend/tests/content-moderation/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
+backend/src/test/java/com/troday/reviews/**
+backend/src/main/java/com/troday/reports/**
+backend/src/test/java/com/troday/reports/**
+backend/docs/contracts/reviews.json
+backend/docs/contracts/reports.json</t>
         </is>
       </c>
       <c r="K41" s="0" t="inlineStr">
@@ -8369,23 +9601,36 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*
-backend/src/modules/account-admin/**
-backend/src/modules/audit/**
-backend/src/modules/admin-dashboard/**
-backend/tests/account-admin/**
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml
+backend/src/main/java/com/troday/accountadmin/**
+backend/src/test/java/com/troday/accountadmin/**
+backend/src/main/java/com/troday/audit/**
+backend/src/test/java/com/troday/audit/**
+backend/src/main/java/com/troday/admindashboard/**
+backend/src/test/java/com/troday/admindashboard/**
+backend/docs/contracts/accountadmin.json
+backend/docs/contracts/audit.json
+backend/docs/contracts/admindashboard.json
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/tests/e2e/release/**</t>
+backend/src/main/resources/application*.yml
+backend/src/test/resources/application-test.yml
+backend/src/test/java/com/troday/e2e/release/**</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -8546,9 +9791,9 @@
       </c>
       <c r="J43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="K43" s="0" t="inlineStr">
@@ -8709,9 +9954,12 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/reviews/**
-backend/src/modules/reports/**
-backend/tests/content-moderation/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
+backend/src/test/java/com/troday/reviews/**
+backend/src/main/java/com/troday/reports/**
+backend/src/test/java/com/troday/reports/**
+backend/docs/contracts/reviews.json
+backend/docs/contracts/reports.json</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -8872,13 +10120,16 @@
       </c>
       <c r="J45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**</t>
         </is>
       </c>
       <c r="K45" s="0" t="inlineStr">
@@ -9039,17 +10290,20 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -9071,7 +10325,7 @@
         <is>
           <t xml:space="preserve">APPROVED valid_until&lt;todayVN → EXPIRED theo chính sách, giữ proof/history.
 Không xóa/ẩn vật lý từng post hoặc kết thúc contract để giả mất quyền.
-Đăng ký worker qua manifest riêng, không sửa worker registry chung.</t>
+Thêm bean @Scheduled trong package houserights; cấu hình lịch qua A, không sửa SchedulingConfig chung.</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -9210,15 +10464,16 @@
       </c>
       <c r="J47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K47" s="0" t="inlineStr">
@@ -9379,15 +10634,16 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -9548,15 +10804,16 @@
       </c>
       <c r="J49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="K49" s="0" t="inlineStr">
@@ -9717,26 +10974,32 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*
-backend/src/modules/posts/**
-backend/tests/posts/**
-backend/contracts/posts.*
-backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*
-backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*
-backend/src/modules/reviews/**
-backend/src/modules/reports/**
-backend/tests/content-moderation/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**
+backend/src/main/java/com/troday/posts/**
+backend/src/test/java/com/troday/posts/**
+backend/docs/contracts/posts.json
+backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**
+backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json
+backend/src/main/java/com/troday/reviews/**
+backend/src/test/java/com/troday/reviews/**
+backend/src/main/java/com/troday/reports/**
+backend/src/test/java/com/troday/reports/**
+backend/docs/contracts/reviews.json
+backend/docs/contracts/reports.json</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -9897,22 +11160,30 @@
       </c>
       <c r="J51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*
-backend/src/modules/billing/**
-backend/tests/billing/**
-backend/contracts/billing.*
-backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml
+backend/src/main/java/com/troday/billing/**
+backend/src/test/java/com/troday/billing/**
+backend/docs/contracts/billing.json
+backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="K51" s="0" t="inlineStr">
@@ -10073,12 +11344,13 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -10242,7 +11514,9 @@
           <t xml:space="preserve">database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/tests/e2e/release/**</t>
+backend/src/main/resources/application*.yml
+backend/src/test/resources/application-test.yml
+backend/src/test/java/com/troday/e2e/release/**</t>
         </is>
       </c>
       <c r="K53" s="0" t="inlineStr">
@@ -22907,7 +24181,7 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khung backend &amp; adapter chung</t>
+          <t xml:space="preserve">Spring Boot &amp; thành phần dùng chung</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -22917,25 +24191,31 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/core/**
-backend/contracts/core.*
-backend/tests/fixtures/A/**
-backend/tests/contracts/A/**
-backend/tests/e2e/platform-*/**
-backend/bootstrap.*
-backend/package*
-backend/lockfile
-.github/workflows/backend-*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
+backend/src/main/java/com/troday/config/**
+backend/src/main/java/com/troday/TrodayApplication.java
+backend/src/test/java/com/troday/shared/**
+backend/src/test/java/com/troday/config/**
+backend/src/test/java/com/troday/support/fixtures/a/**
+backend/src/test/java/com/troday/contract/a/**
+backend/src/test/java/com/troday/e2e/platform/**
+backend/src/test/resources/sql/a/**
+backend/docs/contracts/core.json
+backend/pom.xml
+backend/mvnw
+backend/mvnw.cmd
+backend/.mvn/**
+.github/workflows/backend.yml</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ActorContext, envelope, DB/UoW, procedure runner, idempotency, event/audit ports; không chứa nghiệp vụ nhà/thuê.</t>
+          <t xml:space="preserve">ActorContext, ApiResponse, Spring Security/config, transaction/procedure gateway, idempotency và event/audit ports.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dựng router tự đăng ký manifest module; B/C không cùng sửa một routes.* hoặc DI container.</t>
+          <t xml:space="preserve">A giữ main class/config/POM. B/C thêm bean trong package chức năng, Spring component scan nhận tự động; không có manifest hoặc routes.* chung.</t>
         </is>
       </c>
     </row>
@@ -22952,9 +24232,9 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/identity/**
-backend/tests/identity/**
-backend/contracts/identity.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
+backend/src/test/java/com/troday/identity/**
+backend/docs/contracts/identity.json</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -22981,9 +24261,9 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/files/**
-backend/tests/files/**
-backend/contracts/files.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/files/**
+backend/src/test/java/com/troday/files/**
+backend/docs/contracts/files.json</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -23010,15 +24290,17 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/messaging/**
-backend/src/modules/notifications/**
-backend/tests/messaging/**
-backend/contracts/messaging.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
+backend/src/test/java/com/troday/messaging/**
+backend/src/main/java/com/troday/notifications/**
+backend/src/test/java/com/troday/notifications/**
+backend/docs/contracts/messaging.json
+backend/docs/contracts/notifications.json</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hội thoại, participant, message, notifications, SSE.</t>
+          <t xml:space="preserve">Hội thoại, participant, message, notifications; SSE dùng SseEmitter của Spring MVC.</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -23040,9 +24322,9 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/billing/**
-backend/tests/billing/**
-backend/contracts/billing.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
+backend/src/test/java/com/troday/billing/**
+backend/docs/contracts/billing.json</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -23069,15 +24351,20 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/account-admin/**
-backend/src/modules/audit/**
-backend/src/modules/admin-dashboard/**
-backend/tests/account-admin/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/accountadmin/**
+backend/src/test/java/com/troday/accountadmin/**
+backend/src/main/java/com/troday/audit/**
+backend/src/test/java/com/troday/audit/**
+backend/src/main/java/com/troday/admindashboard/**
+backend/src/test/java/com/troday/admindashboard/**
+backend/docs/contracts/accountadmin.json
+backend/docs/contracts/audit.json
+backend/docs/contracts/admindashboard.json</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khóa phiên/tài khoản, truy vết và tổng quan quản trị; các /admin khác nằm tại module nghiệp vụ của B/C.</t>
+          <t xml:space="preserve">Khóa phiên/tài khoản, truy vết và tổng quan quản trị; các /admin khác nằm tại package nghiệp vụ B/C.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -23099,23 +24386,26 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/properties/**
-backend/src/modules/house-rights/**
-backend/tests/properties/**
-backend/tests/fixtures/B/**
-backend/tests/contracts/B/**
-backend/tests/e2e/property-*/**
-backend/contracts/properties.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
+backend/src/test/java/com/troday/properties/**
+backend/src/main/java/com/troday/houserights/**
+backend/src/test/java/com/troday/houserights/**
+backend/docs/contracts/properties.json
+backend/docs/contracts/houserights.json
+backend/src/test/java/com/troday/support/fixtures/b/**
+backend/src/test/java/com/troday/contract/b/**
+backend/src/test/java/com/troday/e2e/property/**
+backend/src/test/resources/sql/b/**</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhà/phòng, quyền cho thuê, tải phòng, dashboard chủ trọ và các nguồn đọc công khai.</t>
+          <t xml:space="preserve">Nhà/phòng, quyền cho thuê, tải phòng và nguồn đọc công khai.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C chỉ gọi cổng đọc/SQL procedure dưới khóa; không đổi trạng thái phòng bằng setter từ controller.</t>
+          <t xml:space="preserve">C chỉ gọi Java port/SQL procedure dưới khóa; không đổi trạng thái phòng bằng setter từ controller.</t>
         </is>
       </c>
     </row>
@@ -23132,9 +24422,9 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/posts/**
-backend/tests/posts/**
-backend/contracts/posts.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
+backend/src/test/java/com/troday/posts/**
+backend/docs/contracts/posts.json</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -23161,9 +24451,9 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/services/**
-backend/tests/services/**
-backend/contracts/services.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/services/**
+backend/src/test/java/com/troday/services/**
+backend/docs/contracts/services.json</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -23190,10 +24480,10 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/viewings/**
-backend/tests/viewings/**
-backend/tests/e2e/viewing-contract/**
-backend/contracts/viewings.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
+backend/src/test/java/com/troday/viewings/**
+backend/docs/contracts/viewings.json
+backend/src/test/java/com/troday/e2e/viewingcontract/**</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -23220,9 +24510,9 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/roommates/**
-backend/tests/roommates/**
-backend/contracts/roommates.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
+backend/src/test/java/com/troday/roommates/**
+backend/docs/contracts/roommates.json</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -23249,9 +24539,12 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/reviews/**
-backend/src/modules/reports/**
-backend/tests/content-moderation/**</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
+backend/src/test/java/com/troday/reviews/**
+backend/src/main/java/com/troday/reports/**
+backend/src/test/java/com/troday/reports/**
+backend/docs/contracts/reviews.json
+backend/docs/contracts/reports.json</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -23278,22 +24571,23 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/modules/rentals/**
-backend/tests/rentals/**
-backend/tests/fixtures/C/**
-backend/tests/contracts/C/**
-backend/tests/e2e/rental-*/**
-backend/contracts/rentals.*</t>
+          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
+backend/src/test/java/com/troday/rentals/**
+backend/docs/contracts/rentals.json
+backend/src/test/java/com/troday/support/fixtures/c/**
+backend/src/test/java/com/troday/contract/c/**
+backend/src/test/java/com/troday/e2e/rental/**
+backend/src/test/resources/sql/c/**</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contracts, revisions, room_tenants, representative history, join/change requests, templates và liên kết cư dân.</t>
+          <t xml:space="preserve">Contracts, revisions, room_tenants, history, join/change requests, templates và liên kết cư dân; tách package con.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một transaction owner cho toàn bộ vào/rời/đổi phòng; không chia controller và service của cùng luồng cho hai người.</t>
+          <t xml:space="preserve">Một transaction owner cho vào/rời/đổi phòng. Service Java dùng Spring transaction; CALL tự commit dùng gateway riêng.</t>
         </is>
       </c>
     </row>
@@ -23313,17 +24607,17 @@
           <t xml:space="preserve">database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/tests/sql-property/**</t>
+backend/src/test/java/com/troday/sqlproperty/**</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B sửa nguồn thuộc nhà, quota và lịch xem; gửi A tích hợp SQL sinh ra.</t>
+          <t xml:space="preserve">B sửa nguồn nhà, quota và lịch xem; gửi A tích hợp SQL sinh ra.</t>
         </is>
       </c>
       <c r="E15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không tự sửa workflows.sql hoặc bản schema/migration được build.</t>
+          <t xml:space="preserve">Không tự sửa workflows.sql hoặc schema/migration được build.</t>
         </is>
       </c>
     </row>
@@ -23342,24 +24636,24 @@
         <is>
           <t xml:space="preserve">database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/tests/sql-rental/**</t>
+backend/src/test/java/com/troday/sqlrental/**</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C giữ nguồn thuê và file workflows.sql hiện đang chứa nhiều trigger/procedure dùng chung.</t>
+          <t xml:space="preserve">C giữ nguồn thuê và workflows.sql chứa trigger/procedure dùng chung.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A/B cần thay phần của file này thì gửi change request cho C kèm test, không đồng sửa file.</t>
+          <t xml:space="preserve">A/B cần thay file này thì gửi C change request và test, không đồng sửa file.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="72" customHeight="1">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tệp chung &amp; SQL sinh ra</t>
+          <t xml:space="preserve">POM, cấu hình &amp; SQL sinh ra</t>
         </is>
       </c>
       <c r="B17" s="0" t="inlineStr">
@@ -23372,17 +24666,19 @@
           <t xml:space="preserve">database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/tests/e2e/release/**</t>
+backend/src/main/resources/application*.yml
+backend/src/test/resources/application-test.yml
+backend/src/test/java/com/troday/e2e/release/**</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">A cấp thứ tự migration, build/commit output SQL, khóa phiên bản dependency và CI.</t>
+          <t xml:space="preserve">A cấp thứ tự migration, build SQL, tích hợp cấu hình Spring, phiên bản dependency và CI.</t>
         </is>
       </c>
       <c r="E17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">B/C có thể chạy build trong thư mục tạm để test; A tái sinh output trên nhánh tích hợp từ toàn bộ nguồn mới nhất.</t>
+          <t xml:space="preserve">Không tự tạo schema từ ORM; A tái sinh output SQL và duyệt thay đổi cấu hình chung trong lượt bàn giao.</t>
         </is>
       </c>
     </row>
@@ -23849,17 +25145,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ActorContext; ResultEnvelope; DomainError; UnitOfWork; ProcedureRunner</t>
+          <t xml:space="preserve">ActorContext; ApiResponse&lt;T&gt;; DomainException; TransactionTemplate; StoredProcedureGateway</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">actor.userId/roles/sessionId/requestId; ID string; decimal/date; UoW(connection) hoặc CALL tự transaction</t>
+          <t xml:space="preserve">SecurityContext → actor.userId/roles/sessionId/requestId; ID string; BigDecimal/Instant/LocalDate</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không tin actor trong body; CALL không chạy bên trong transaction app.</t>
+          <t xml:space="preserve">Service dùng transaction Spring; CALL tự commit qua bean Propagation.NEVER, không self-invocation. tx trong các port là ngữ cảnh cùng DataSource trên server, không truyền JDBC Connection qua HTTP.</t>
         </is>
       </c>
       <c r="H2" s="2" t="str">
@@ -23900,7 +25196,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C mở UoW khi liên kết; adapter A dùng cùng tx, không gọi HTTP hoặc commit riêng.</t>
+          <t xml:space="preserve">Service C mở transaction Spring khi liên kết; adapter A tham gia cùng tx/DataSource, không gọi HTTP hoặc commit riêng.</t>
         </is>
       </c>
       <c r="H3" s="0" t="str">

</xml_diff>

<commit_message>
docs: align backend plan with layered structure and shared preparation
</commit_message>
<xml_diff>
--- a/docs/backend-team-checklist.xlsx
+++ b/docs/backend-team-checklist.xlsx
@@ -162,7 +162,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">52 task chạy TUẦN TỰ theo STT chung 01–52, mỗi lần một task; A/B/C giữ owner theo module. Bao phủ 176 API. FE/AI trống. Đây là kế hoạch, chưa có backend nào được triển khai.</t>
+          <t xml:space="preserve">52 task chạy TUẦN TỰ theo STT chung 01–52, mỗi lần một task; A/B/C phụ trách chức năng, thư mục Java theo tầng tại troday/BE. Bao phủ 176 API. FE/AI trống. Lớp nghiệp vụ được triển khai theo task.</t>
         </is>
       </c>
     </row>
@@ -234,7 +234,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điền tên thành viên tương ứng A/B/C tại Tong_quan, cột Tên thực tế; giữ ký hiệu owner để liên kết task/API ổn định. Không đổi owner của một task lẻ rồi cùng sửa một module.</t>
+          <t xml:space="preserve">Điền tên thành viên tương ứng A/B/C tại Tong_quan, cột Tên thực tế; giữ ký hiệu owner để liên kết task/API ổn định. Không đổi owner của một task lẻ rồi cùng sửa các lớp của một chức năng.</t>
         </is>
       </c>
     </row>
@@ -270,7 +270,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Java 21 LTS + Spring Boot + Maven Wrapper + MySQL; Spring JDBC tích hợp SQL/procedure hiện có. BE-A01 tạo project thật. Sheet Cau_truc_BE mô tả stack, cây thư mục và quy ước.</t>
+          <t xml:space="preserve">Java 21 LTS + Spring Boot + Maven Wrapper + MySQL; Spring JDBC tích hợp SQL/procedure hiện có. Khung backend đã có tại troday/BE. Sheet Cau_truc_BE mô tả stack, cây thư mục và quy ước.</t>
         </is>
       </c>
     </row>
@@ -282,7 +282,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A tích hợp TrodayApplication/config/shared/pom.xml/Maven Wrapper/application*.yml/CI/output SQL ngay trong lượt bàn giao cần nó. B/C thêm bean trong package chức năng và sửa source SQL đã phân. backend/** là bố cục đề xuất, chưa phải backend đã có.</t>
+          <t xml:space="preserve">A tích hợp main class, config/security/exception/util, DTO chung, POM/Wrapper, profile, CI và output SQL. Mỗi người giữ các lớp nghiệp vụ của mình trong controller/service/repository/model/dto. Fixture Java/SQL đặt tên theo chức năng trong thư mục dùng chung.</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B94"/>
+  <dimension ref="A1:B118"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Java Spring Boot dự kiến</t>
+          <t xml:space="preserve">Java Spring Boot theo tầng</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã chốt stack cho kế hoạch; repo chưa có ứng dụng Java Spring Boot chạy thật. BE-A01 mới tạo pom.xml, main class và cấu hình.</t>
+          <t xml:space="preserve">Khung Spring Boot đã có tại troday/BE, tổ chức package theo tầng. Các API nghiệp vụ và lớp mẫu bên dưới sẽ được triển khai theo từng task; tiến độ chỉ được xác nhận bằng checklist và bàn giao.</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">BE-A01 chọn bản Spring Boot stable tương thích Java 21 và dependency của dự án, pin version trong pom.xml/Maven Wrapper. Không dùng SNAPSHOT; chưa có pom.xml thực tế để xác nhận patch version.</t>
+          <t xml:space="preserve">BE/pom.xml hiện pin Spring Boot 3.5.16, Java release 21; Maven Wrapper 3.3.4 dùng Maven 3.9.9. A quản lý phiên bản dependency và cấu hình build, kiểm tra tương thích khi nâng cấp.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/                                      # Dự án Spring Boot dự kiến; chưa tạo</t>
+          <t xml:space="preserve">troday/</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── pom.xml                                   # A: version, dependency và Maven plugins</t>
+          <t xml:space="preserve">├── BE/                                       # Backend Spring Boot, package theo tầng</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── mvnw / mvnw.cmd / .mvn/wrapper/            # A: cùng một Maven Wrapper cho team</t>
+          <t xml:space="preserve">│   ├── pom.xml                               # A: version, dependency và Maven plugins</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── docs/contracts/                           # JSON/schema API; mỗi module có file riêng</t>
+          <t xml:space="preserve">│   ├── mvnw / mvnw.cmd / .mvn/wrapper/        # Maven Wrapper dùng chung</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── core.json                             # A: envelope/error/type conventions</t>
+          <t xml:space="preserve">│   ├── docs/contracts/                       # JSON/schema theo endpoint hoặc tài nguyên</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── identity.json, files.json, messaging.json, notifications.json, billing.json # A</t>
+          <t xml:space="preserve">│   ├── src/main/java/com/troday/</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── accountadmin.json, audit.json, admindashboard.json       # A</t>
+          <t xml:space="preserve">│   │   ├── TrodayApplication.java            # A: @SpringBootApplication ở package gốc</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── properties.json, houserights.json, posts.json, services.json, viewings.json # B</t>
+          <t xml:space="preserve">│   │   ├── config/                          # A: cấu hình bean, SecurityConfig, DataSource</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── roommates.json, reviews.json, reports.json               # B</t>
+          <t xml:space="preserve">│   │   ├── controller/                      # REST controller của mọi chức năng</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   └── rentals.json                          # C</t>
+          <t xml:space="preserve">│   │   ├── dto/</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── src/main/java/com/troday/</t>
+          <t xml:space="preserve">│   │   │   ├── request/                     # Request DTO và validation</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── TrodayApplication.java                # A: @SpringBootApplication ở package gốc</t>
+          <t xml:space="preserve">│   │   │   └── response/                    # Response DTO, ApiResponse, PageMeta</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── config/                              # A: Security/DataSource/Scheduling config</t>
+          <t xml:space="preserve">│   │   ├── exception/                       # DomainException, GlobalExceptionHandler</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── shared/                              # A: code dùng chung, không chứa nghiệp vụ thuê</t>
+          <t xml:space="preserve">│   │   ├── integration/                     # Client/gateway tới dịch vụ bên ngoài</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── api/                             # ApiResponse, PageMeta, RequestId</t>
+          <t xml:space="preserve">│   │   ├── model/                           # Model Java thuần dùng với Spring JDBC</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── error/                           # GlobalExceptionHandler, DomainException</t>
+          <t xml:space="preserve">│   │   ├── repository/                      # SQL/CRUD và implementation cổng đọc</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── security/                        # ActorContext, scope helpers</t>
+          <t xml:space="preserve">│   │   │   ├── mapper/                     # JDBC RowMapper</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── transaction/                     # StoredProcedureGateway, transaction helpers</t>
+          <t xml:space="preserve">│   │   │   └── procedure/                  # Gateway gọi stored procedure</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── audit/                           # AuditPort/adapter, target D14</t>
+          <t xml:space="preserve">│   │   ├── security/                        # ActorContext, xác thực, phân quyền</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── event/                           # EventPort/outbox adapter</t>
+          <t xml:space="preserve">│   │   ├── service/                         # Nghiệp vụ, interface bàn giao, transaction</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   ├── idempotency/                     # request key/hash/result store</t>
+          <t xml:space="preserve">│   │   └── util/                            # Hàm tiện ích, thời gian, định dạng</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   │   └── time/                            # UTC Instant / ngày nghiệp vụ Việt Nam</t>
+          <t xml:space="preserve">│   ├── src/main/resources/</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── identity/                            # A: tài khoản, phiên, OTP, xác minh</t>
+          <t xml:space="preserve">│   │   ├── application.yml                  # A: cấu hình chung qua environment</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── files/                               # A: kho tệp, private access, retention</t>
+          <t xml:space="preserve">│   │   └── application-local.yml            # Profile local; không commit secret</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── messaging/                           # A: conversation/messages/post share</t>
+          <t xml:space="preserve">│   ├── src/test/java/com/troday/</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── notifications/                       # A: feed, read-state, SSE</t>
+          <t xml:space="preserve">│   │   ├── TrodayApplicationTests.java       # Smoke test context và Security</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── billing/                             # A: invoices/invoice_items</t>
+          <t xml:space="preserve">│   │   ├── config/ controller/ exception/ repository/ security/ service/</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── accountadmin/ audit/ admindashboard/  # A: user lock, audit query, tổng quan</t>
+          <t xml:space="preserve">│   │   ├── integration/                     # Test tích hợp, MySQL/procedure/race</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── properties/ houserights/              # B: nhà/phòng, quyền cho thuê</t>
+          <t xml:space="preserve">│   │   ├── contract/                        # Contract test theo endpoint/tài nguyên</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── posts/ services/ viewings/            # B: tin, giá dịch vụ, lịch xem</t>
+          <t xml:space="preserve">│   │   ├── e2e/                             # Test luồng nghiệp vụ xuyên suốt</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── roommates/ reviews/ reports/          # B: kết nối/ghép, đánh giá/báo cáo</t>
+          <t xml:space="preserve">│   │   └── support/fixtures/                # Fixture đặt tên theo chức năng</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   └── rentals/                             # C: mỗi nhóm thuê có package con</t>
+          <t xml:space="preserve">│   ├── src/test/resources/</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│       ├── contracts/ revisions/ residents/</t>
+          <t xml:space="preserve">│   │   ├── application-test.yml             # Profile test</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│       ├── joins/ changes/ representatives/</t>
+          <t xml:space="preserve">│   │   └── sql/                            # SQL fixture đặt tên theo chức năng</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│       └── templates/ residencylink/ port/</t>
+          <t xml:space="preserve">│   └── target/                              # Maven sinh ra; không commit</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── src/main/resources/</t>
+          <t xml:space="preserve">└── database/</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── application.yml                      # A: cấu hình chung, giá trị qua environment</t>
+          <t xml:space="preserve">    ├── source/                              # SQL nguồn do owner bàn giao</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   └── application-local.yml                # A: profile local; không commit secret</t>
+          <t xml:space="preserve">    └── migrations/                          # A tích hợp migration đã review</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── src/test/java/com/troday/</t>
+          <t xml:space="preserve">SQL nguồn hiện có: wireframe/room_rental_wireframe_v5/database/.</t>
         </is>
       </c>
     </row>
@@ -1607,525 +1607,973 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── shared/ config/                      # A: core/config tests</t>
+          <t xml:space="preserve">A tích hợp SQL đã review vào troday/database theo task; không tự sinh schema từ ORM.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="72" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── identity/ files/ messaging/ notifications/ billing/  # A</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/                  # Ví dụ lớp nhà/phòng của B</t>
         </is>
       </c>
     </row>
     <row r="53" ht="72" customHeight="1">
       <c r="A53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── properties/ services/ posts/ viewings/ roommates/   # B</t>
+          <t xml:space="preserve">├── controller/HouseController.java           # @RestController, HTTP/DTO/scope</t>
         </is>
       </c>
     </row>
     <row r="54" ht="72" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── houserights/ reviews/ reports/ sqlproperty/ # B</t>
+          <t xml:space="preserve">├── dto/request/CreateHouseRequest.java       # record + jakarta.validation</t>
         </is>
       </c>
     </row>
     <row r="55" ht="72" customHeight="1">
       <c r="A55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── accountadmin/ audit/ admindashboard/   # A</t>
+          <t xml:space="preserve">├── dto/response/HouseResponse.java            # Response riêng</t>
         </is>
       </c>
     </row>
     <row r="56" ht="72" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── sqlrental/                           # C: procedure/trigger tests</t>
+          <t xml:space="preserve">├── service/HouseService.java                 # @Service, quy tắc và điều phối</t>
         </is>
       </c>
     </row>
     <row r="57" ht="72" customHeight="1">
       <c r="A57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── rentals/                             # C: contract/occupancy/race tests</t>
+          <t xml:space="preserve">├── service/PropertyReadPort.java             # Interface bàn giao cho A/C</t>
         </is>
       </c>
     </row>
     <row r="58" ht="72" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── support/fixtures/a/ b/ c/             # Fixture Java riêng theo owner</t>
+          <t xml:space="preserve">├── repository/HouseRepository.java           # @Repository, SQL/DB mapping</t>
         </is>
       </c>
     </row>
     <row r="59" ht="72" customHeight="1">
       <c r="A59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── contract/a/ b/ c/                     # Contract tests riêng</t>
+          <t xml:space="preserve">├── repository/PropertyReadRepository.java    # Implementation cổng đọc độc lập</t>
         </is>
       </c>
     </row>
     <row r="60" ht="72" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   └── e2e/platform/ property/ viewingcontract/ rental/ release/</t>
+          <t xml:space="preserve">├── repository/mapper/HouseRowMapper.java     # JDBC RowMapper</t>
         </is>
       </c>
     </row>
     <row r="61" ht="72" customHeight="1">
       <c r="A61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── src/test/resources/</t>
+          <t xml:space="preserve">└── model/House.java                          # Model Java thuần</t>
         </is>
       </c>
     </row>
     <row r="62" ht="72" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   ├── application-test.yml                 # A: MySQL/kho tệp test độc lập</t>
+          <t xml:space="preserve">Controller → Service → Repository / Procedure gateway → MySQL</t>
         </is>
       </c>
     </row>
     <row r="63" ht="72" customHeight="1">
       <c r="A63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">│   └── sql/a/ b/ c/                         # SQL fixture theo owner</t>
+          <t xml:space="preserve">Interface bàn giao đặt trong service/; implementation đọc đặt trong repository/.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="72" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Ví dụ lớp theo tầng</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">└── target/                                  # Maven sinh ra; không commit</t>
+          <t xml:space="preserve">Đây là ví dụ tên lớp sẽ triển khai, không phải các lớp nghiệp vụ đã có.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="72" customHeight="1">
       <c r="A65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Đề xuất phần dùng chung</t>
         </is>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">database/source/*.sql                         # Nguồn SQL hiện có ở root repo: B/C theo owner</t>
+          <t xml:space="preserve">Làm nền tảng chung trước; sau đó chuẩn bị model, mapper và repository vừa đủ cho từng nhóm chức năng rồi viết service của nhóm đó. Đây là thứ tự chi tiết bên trong các task hiện có.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="72" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cây thư mục BE</t>
+          <t xml:space="preserve">Phạm vi chuẩn bị</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">database/schema.sql + migrations/               # A tích hợp output; không tự sinh schema từ ORM</t>
+          <t xml:space="preserve">Bước 1–2 chuẩn bị nền tảng; bước 3–6 lặp lại cho từng nhóm chức năng theo hàng đợi. Các model/repository của toàn hệ thống không phải điều kiện để bắt đầu AuthService hay HouseService.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="72" customHeight="1">
       <c r="A67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 01: Chốt hợp đồng dữ liệu</t>
         </is>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">com/troday/properties/                        # Ví dụ một module của B</t>
+          <t xml:space="preserve">Phụ trách: A + B + C
+Thống nhất field/nullable/status từ SQL, ID JSON, tiền, thời gian, lỗi, phân trang và chữ ký hàm. Ghi consumer của từng model/query.
+Điều kiện: B01/C01 bàn giao phân tích; A02 chốt contract trước các consumer.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="72" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 02: Hoàn tất nền tảng dùng chung</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── controller/HouseController.java            # @RestController, chỉ HTTP/DTO/scope</t>
+          <t xml:space="preserve">Phụ trách: A
+ApiResponse/PageMeta, lỗi tập trung, ActorContext, Clock, cấu hình JDBC và quy ước transaction/procedure.
+Điều kiện: A01/A02 có code và test; model và query nghiệp vụ chưa cần hoàn tất toàn bộ.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="72" customHeight="1">
       <c r="A69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 03: Model/projection cho nhóm đang làm</t>
         </is>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── dto/request/CreateHouseRequest.java        # record + jakarta.validation</t>
+          <t xml:space="preserve">Phụ trách: Owner chức năng
+Chỉ tạo model được luồng hiện tại hoặc consumer đã xác định sử dụng; tách projection đọc khỏi response HTTP có dữ liệu riêng tư.
+Điều kiện: Có danh sách field và nơi sử dụng; không sinh model cho mọi bảng chỉ để đủ bộ.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="72" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 04: RowMapper và repository/query</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── dto/response/HouseResponse.java            # Không trả domain model trực tiếp</t>
+          <t xml:space="preserve">Phụ trách: Owner chức năng
+mapRow, truy vấn cụ thể, lọc quyền, null/decimal/date mapping, ghi có điều kiện. Luồng SQL đã có procedure dùng gateway thay CRUD chồng lên procedure.
+Điều kiện: Truy vấn/ghi chạy trên MySQL test, xử lý trường hợp không có dữ liệu và lỗi ràng buộc.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="72" customHeight="1">
       <c r="A71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 05: Bàn giao hàm được nhiều luồng dùng</t>
         </is>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── service/HouseService.java                  # @Service, quy tắc và điều phối</t>
+          <t xml:space="preserve">Phụ trách: Provider A/B/C
+Cổng tệp/token/audit/event, snapshot phòng/cư trú, báo giá dịch vụ và bằng chứng lịch xem theo mốc cung cấp bên dưới.
+Điều kiện: Có implementation và test; interface hoặc mock riêng lẻ chưa phải bàn giao hoàn tất.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="72" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">Bước 06: Service → controller → kiểm thử luồng</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── repository/HouseRepository.java            # @Repository, SQL/DB mapping</t>
+          <t xml:space="preserve">Phụ trách: Owner chức năng
+Service điều phối quyền/trạng thái/transaction; controller nhận DTO và trả kết quả. Hoàn tất một luồng có thể kiểm thử rồi bổ sung nhóm tiếp theo.
+Điều kiện: Kiểm thử thành công, sai quyền, dữ liệu cũ, rollback và retry liên quan; ghi PR/test vào task hiện tại.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="72" customHeight="1">
       <c r="A73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-01 — Response, lỗi và phân trang</t>
         </is>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── repository/mapper/HouseRowMapper.java      # RowMapper dùng JDBC</t>
+          <t xml:space="preserve">Phạm vi: Toàn hệ thống
+Provider: A / BE-A02
+File dưới BE/src/main/java/com/troday/:
+dto/response/ApiResponse.java
+dto/response/PageMeta.java
+dto/request/PageQuery.java
+exception/DomainException.java
+exception/GlobalExceptionHandler.java
+Hàm minh họa:
+ApiResponse.success(data)
+PageQuery.validate(allowedSortFields)
+GlobalExceptionHandler.handleDomainException(...)
+Consumer: BE-A03, BE-B02, BE-C02
+Nghiệm thu: Contract JSON đúng kiểu; validate page/size/sort, thống nhất lỗi và requestId; không lộ SQL hoặc PII.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="72" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-02 — Actor, đồng hồ và ranh giới giao dịch</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── domain/House.java                          # Model Java thuần, chưa yêu cầu @Entity</t>
+          <t xml:space="preserve">Phạm vi: Toàn hệ thống
+Provider: A / BE-A02
+File dưới BE/src/main/java/com/troday/:
+security/ActorContext.java
+config/ClockConfig.java
+exception/ProcedureErrorTranslator.java
+repository/procedure/StoredProcedureGateway.java
+Hàm minh họa:
+ActorContext.requireUserId()
+Clock.instant()
+ProcedureErrorTranslator.toDomainException(sqlException)
+StoredProcedureGateway: kiểm tra Propagation.NEVER qua Spring proxy
+Consumer: BE-A03, BE-B02, BE-C04
+Nghiệm thu: Actor từ SecurityContext; Clock có thể cố định trong test. Gateway dùng chữ ký procedure tường minh, không cho client chọn SQL/procedure tùy ý.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="72" customHeight="1">
       <c r="A75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-03 — Dữ liệu người dùng và phiên</t>
         </is>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">├── port/PropertyReadPort.java                 # Interface công khai cho consumer</t>
+          <t xml:space="preserve">Phạm vi: Nhiều luồng danh tính
+Provider: A / BE-A03
+File dưới BE/src/main/java/com/troday/:
+model/User.java
+model/AuthSession.java
+repository/mapper/UserRowMapper.java
+repository/UserRepository.java
+repository/SessionRepository.java
+Hàm minh họa:
+UserRepository.findById(userId)
+UserRepository.findByLogin(login)
+SessionRepository.findActive(sessionId,now)
+Consumer: BE-A03, BE-A06, BE-A07
+Nghiệm thu: Chuẩn bị trong A03 trước AuthService. Thông tin xác thực không đi vào response chung; kiểm tra user/session bị khóa hoặc hết hạn.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="72" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-04 — Idempotency, audit và sự kiện</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">└── adapter/PropertyReadJdbcAdapter.java        # Bean đọc riêng, tránh vòng phụ thuộc service</t>
+          <t xml:space="preserve">Phạm vi: Các luồng có tác dụng ghi
+Provider: A / BE-A04
+File dưới BE/src/main/java/com/troday/:
+repository/IdempotencyRepository.java
+service/IdempotencyService.java
+service/AuditPort.java
+service/EventPort.java
+Hàm minh họa:
+IdempotencyRepository.tryStart(scope,key,hash)
+IdempotencyRepository.storeResult(...)
+AuditPort.append(tx,...)
+EventPort.append(tx,event)
+Consumer: BE-A05, BE-B06, BE-C03
+Nghiệm thu: Cùng key/payload không ghi lặp; khác payload bị từ chối. Audit/event dùng đúng transaction; procedure đã ghi thì không ghi lần hai. D09/D14 phải chốt.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="72" customHeight="1">
       <c r="A77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-05 — Metadata tệp và quyền sử dụng</t>
         </is>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controller → Service → Repository / Procedure adapter → MySQL</t>
+          <t xml:space="preserve">Phạm vi: Xác minh, tin đăng, chứng cứ
+Provider: A / BE-A05
+File dưới BE/src/main/java/com/troday/:
+model/FileMetadata.java
+repository/mapper/FileMetadataRowMapper.java
+repository/FileRepository.java
+service/FilePort.java
+integration/FileStorageClient.java
+Hàm minh họa:
+FileRepository.findById(fileId)
+FilePort.assertUsable(actor,fileId,purpose,context,tx)
+FilePort.authorizeDownload(...)
+Consumer: BE-A06, BE-B05, BE-B06, BE-C13
+Nghiệm thu: Kiểm thử quyền đọc private, chủ sở hữu, mục đích, trạng thái tệp và retention; trả metadata cần thiết, không dùng URL bucket cố định.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="72" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một module mẫu</t>
+          <t xml:space="preserve">COMMON-06 — Token dùng một lần</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consumer module → Java Port interface → Adapter của module provider</t>
+          <t xml:space="preserve">Phạm vi: OTP/reset và liên kết cư dân
+Provider: A / BE-A07
+File dưới BE/src/main/java/com/troday/:
+repository/TokenRepository.java
+service/TokenPort.java
+Hàm minh họa:
+TokenPort.issue(purpose,target,actor,tx)
+TokenPort.consume(purpose,target,actor,tx)
+Consumer: BE-A07, BE-C08
+Nghiệm thu: Consume nguyên tử, đúng purpose/target, có hạn dùng; rollback luồng liên kết phải rollback consume. Không tự commit ngoài transaction consumer.</t>
         </is>
       </c>
     </row>
     <row r="79" ht="72" customHeight="1">
       <c r="A79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main class và package</t>
+          <t xml:space="preserve">COMMON-07 — Nhà/phòng và mapper cơ bản</t>
         </is>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đặt TrodayApplication trong com.troday, các package chức năng nằm bên dưới. Package viết thường, không có dấu gạch nối; dùng houserights/accountadmin thay house-rights/account-admin. Đây là quy ước của team, không phải cấu trúc duy nhất Spring Boot cho phép.</t>
+          <t xml:space="preserve">Phạm vi: CRUD và nguồn đọc phòng
+Provider: B / BE-B02
+File dưới BE/src/main/java/com/troday/:
+model/House.java
+model/Room.java
+repository/mapper/HouseRowMapper.java
+repository/mapper/RoomRowMapper.java
+repository/HouseRepository.java
+repository/RoomRepository.java
+Hàm minh họa:
+HouseRepository.findOwnedById(actor,houseId)
+RoomRepository.findById(roomId)
+HouseRepository.insert(...)
+Consumer: BE-B02, BE-B04
+Nghiệm thu: Làm model/mapper/repository trong B02 trước HouseService/RoomService; quyền sửa nhà và xử lý sức chứa đúng SQL hiện có.</t>
         </is>
       </c>
     </row>
     <row r="80" ht="72" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bean và route theo module</t>
+          <t xml:space="preserve">COMMON-08 — Báo giá dịch vụ hiệu lực</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controller dùng @RestController/@RequestMapping, nghiệp vụ @Service, SQL adapter @Repository; constructor injection. Spring component scan nhận bean dưới package gốc, không có file routes.* hoặc manifest module để ba người cùng sửa.</t>
+          <t xml:space="preserve">Phạm vi: Dịch vụ và hóa đơn
+Provider: B / BE-B03
+File dưới BE/src/main/java/com/troday/:
+model/ServiceQuote.java
+repository/mapper/ServiceQuoteRowMapper.java
+repository/ServiceQuoteRepository.java
+service/ServiceQuotePort.java
+Hàm minh họa:
+ServiceQuoteRepository.findEffectiveByRoomId(roomId)
+ServiceQuotePort.getEffective(roomId,tx)
+Consumer: BE-B03, BE-A10
+Nghiệm thu: Null kế thừa, override 0 giữ 0, tiền dùng BigDecimal; invoice giữ snapshot, không đọc lại giá mới thay giá đã chốt.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="72" customHeight="1">
       <c r="A81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">DTO, kiểu số và ngày</t>
+          <t xml:space="preserve">COMMON-09 — Snapshot phòng và kết nối</t>
         </is>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Request/response DTO riêng, có @Valid và Bean Validation. Tiền dùng BigDecimal; ID trong JSON giữ chuỗi như đặc tả; Instant cho thời điểm UTC, LocalDate cho ngày Việt Nam. Không tự expose model hoặc giấy tờ cá nhân.</t>
+          <t xml:space="preserve">Phạm vi: Chat, lịch xem và hợp đồng
+Provider: B / BE-B04
+File dưới BE/src/main/java/com/troday/:
+model/RoomSnapshot.java
+repository/mapper/RoomSnapshotRowMapper.java
+repository/PropertyReadRepository.java
+repository/ConnectionReadRepository.java
+service/PropertyReadPort.java
+service/ConnectionReadPort.java
+Hàm minh họa:
+PropertyReadPort.getRentalSnapshot(actor,roomId,tx)
+ConnectionReadPort.assertAccepted(actor,connectionId,tx)
+Consumer: BE-A08, BE-C05
+Nghiệm thu: Provider SQL thật, không có PII cư dân. Snapshot dùng đọc; giữ phòng/gia hạn/chuyển vẫn kiểm tra lại quyền và capacity dưới khóa.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="72" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giao dịch do service quản lý</t>
+          <t xml:space="preserve">COMMON-10 — Snapshot hợp đồng và cư trú</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dùng @Transactional tại service public hoặc TransactionTemplate cho thao tác tự ghi nhiều bảng. Các repository/port dùng cùng DataSource và transaction Spring; không commit riêng trong adapter. Tham số tx trong đặc tả là ngữ cảnh server, không truyền JDBC Connection qua HTTP.</t>
+          <t xml:space="preserve">Phạm vi: Hồ sơ ở ghép, hóa đơn, thuê
+Provider: C / BE-C02
+File dưới BE/src/main/java/com/troday/:
+model/ContractSnapshot.java
+model/ActiveStay.java
+repository/mapper/ContractSnapshotRowMapper.java
+repository/ResidencyReadRepository.java
+service/ResidencyReadPort.java
+Hàm minh họa:
+ResidencyReadPort.getContractSnapshot(actor,contractId,tx)
+ResidencyReadPort.getActiveStay(actor,tx)
+ResidencyReadPort.getMetrics(...)
+Consumer: BE-C05, BE-B11, BE-A10
+Nghiệm thu: Kiểm thử bằng MySQL fixture trước API tạo hợp đồng; phân biệt ACTIVE/PLANNED, payer và representative; chỉ trả projection được phép đọc.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="72" customHeight="1">
       <c r="A83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giao dịch do procedure quản lý</t>
+          <t xml:space="preserve">COMMON-11 — Gateway giao dịch thuê và revision</t>
         </is>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">StoredProcedureGateway là bean riêng, gọi SimpleJdbcCall/CallableStatement với tham số IN/OUT tường minh. Dùng Propagation.NEVER để fail nếu caller đang có transaction Spring; không bọc CALL tự START/COMMIT trong @Transactional. Test đường gọi qua proxy, không self-invocation bỏ qua guard.</t>
+          <t xml:space="preserve">Phạm vi: Các luồng ghi thuê
+Provider: C / BE-C04
+File dưới BE/src/main/java/com/troday/:
+repository/procedure/RentalProcedureGateway.java
+Hàm minh họa:
+RentalProcedureGateway: CALL có IN/OUT và expectedRevision theo từng thủ tục
+Dùng ProcedureErrorTranslator của A; C bàn giao mã SIGNAL và tình huống nghiệp vụ cần ánh xạ
+Consumer: BE-C05, BE-C06, BE-C07
+Nghiệm thu: C04 bàn giao nền gọi procedure và bảo vệ revision; từng hàm CALL được hoàn thiện ở task luồng tương ứng. Không bọc CALL tự commit trong transaction Spring; test lỗi/rollback/race tại task sử dụng.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="72" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tôn trọng SQL hiện có</t>
+          <t xml:space="preserve">COMMON-12 — Bằng chứng và timeline lịch xem</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MySQL CHECK/FK/trigger và thủ tục là nguồn ràng buộc đã có. Kế hoạch chọn Spring JDBC để tích hợp; không bật Hibernate ddl-auto=create/update hoặc tạo bản entity DDL khác. Nếu bổ sung JPA sau này phải có quyết định riêng về mapping và transaction.</t>
+          <t xml:space="preserve">Phạm vi: Chat và tạo hợp đồng
+Provider: B / BE-B08
+File dưới BE/src/main/java/com/troday/:
+model/ViewingEvidence.java
+repository/ViewingReadRepository.java
+service/ViewingReadPort.java
+Hàm minh họa:
+ViewingReadPort.getTimeline(actor,context,tx)
+ViewingReadPort.getRentalEvidence(actor,context,tx)
+Consumer: BE-A11, BE-C05
+Nghiệm thu: Hoàn tất provider trong B08 trước C05; dữ liệu gốc của lịch, đúng tenant/landlord và trạng thái hiện tại, không sao chép trạng thái từ chat.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="72" customHeight="1">
       <c r="A85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Không tạo vòng phụ thuộc bean</t>
+          <t xml:space="preserve">BE-A03 — AuthService.login(...)</t>
         </is>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Port đọc được implement bằng adapter/repository riêng; không inject ngược service nghiệp vụ vào nhau và không dùng @Lazy để che vòng phụ thuộc. Test @SpringBootTest phải khởi tạo được application context.</t>
+          <t xml:space="preserve">Đầu vào: COMMON-01, COMMON-02, COMMON-03
+Validate → tìm User → kiểm tra password/trạng thái → tạo Session → trả DTO.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="72" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test và cấu hình dùng chung</t>
+          <t xml:space="preserve">BE-A05 — FileService.completeUpload(...)</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">JUnit/MockMvc kiểm thử HTTP/security; MySQL test độc lập kiểm thử procedure/race/rollback. A giữ pom.xml, wrapper, main class, config dùng chung và resources profile; B/C giữ package chức năng, test và contract riêng. Lệnh Maven chỉ chạy được sau khi BE-A01 tạo dự án.</t>
+          <t xml:space="preserve">Đầu vào: COMMON-01, COMMON-02, COMMON-04, COMMON-05
+Kiểm tra actor/purpose → xác minh object/MIME/hash → cập nhật metadata → ghi audit/event → trả DTO.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="72" customHeight="1">
       <c r="A87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chạy local sau BE-A01</t>
+          <t xml:space="preserve">BE-B02 — HouseService.createHouse(...)</t>
         </is>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">.\mvnw.cmd spring-boot:run "-Dspring-boot.run.profiles=local"
-Đã cấu hình MySQL local và biến môi trường.</t>
+          <t xml:space="preserve">Đầu vào: COMMON-01, COMMON-02, COMMON-04, COMMON-07
+Validate/quyền chủ trọ → ghi nhà/phòng theo transaction đã chốt → audit/event → trả DTO.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="72" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit/controller tests</t>
+          <t xml:space="preserve">BE-C05 — ContractService.submit(...)</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">.\mvnw.cmd test
-JUnit Jupiter / MockMvc; không dùng DB thật.</t>
+          <t xml:space="preserve">Đầu vào: COMMON-02, COMMON-04, COMMON-09, COMMON-10, COMMON-11, COMMON-12
+Kiểm tra actor/bằng chứng xem → đọc snapshot → CALL tạo hợp đồng và kiểm tra lại dưới khóa → đọc kết quả; không bọc procedure tự commit trong transaction Spring.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="72" customHeight="1">
       <c r="A89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm thử/bản build tích hợp</t>
+          <t xml:space="preserve">BE-A10 — InvoiceService.createDraft(...)</t>
         </is>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">.\mvnw.cmd verify
-BE-A01 cấu hình integration tests và DB MySQL test riêng.</t>
+          <t xml:space="preserve">Đầu vào: COMMON-01, COMMON-02, COMMON-04, COMMON-08, COMMON-10
+Đọc cư trú/người trả → lấy báo giá → tính tiền → lưu invoice/items và snapshot trong cùng transaction.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="72" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Linux/macOS</t>
+          <t xml:space="preserve">Điều kiện bắt đầu service</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">./mvnw test
-Dùng ./mvnw verify khi kiểm thử tích hợp.</t>
+          <t xml:space="preserve">Chữ ký hàm, đầu vào/đầu ra, field nullable và người sở hữu đã được chốt cho luồng đang viết.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="72" customHeight="1">
       <c r="A91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spring Boot: bố trí main class và package</t>
+          <t xml:space="preserve">Điều kiện bắt đầu service</t>
         </is>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://docs.spring.io/spring-boot/reference/using/structuring-your-code.html</t>
+          <t xml:space="preserve">Model/RowMapper/query mà luồng dùng có test phù hợp; repository không chỉ là interface hoặc mock.</t>
         </is>
       </c>
     </row>
     <row r="92" ht="72" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spring JDBC: SimpleJdbcCall</t>
+          <t xml:space="preserve">Điều kiện bắt đầu service</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://docs.spring.io/spring-framework/reference/data-access/jdbc/simple.html</t>
+          <t xml:space="preserve">Quyền theo actor/tài nguyên, trạng thái và thời điểm cần kiểm tra lại dưới khóa đã rõ.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="72" customHeight="1">
       <c r="A93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spring: Propagation.NEVER</t>
+          <t xml:space="preserve">Điều kiện bắt đầu service</t>
         </is>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://docs.spring.io/spring-framework/docs/current/javadoc-api/org/springframework/transaction/annotation/Propagation.html</t>
+          <t xml:space="preserve">Đã chọn một chủ transaction: service Spring hoặc procedure tự quản lý; audit/event/token tham gia đúng ranh giới.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="72" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Điều kiện bắt đầu service</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Có ca thành công và các ca sai quyền, không tìm thấy, dữ liệu cũ, rollback/retry cần cho luồng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="72" customHeight="1">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giới hạn cách chia</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không cần BaseRepository&lt;T&gt;/BaseService&lt;T&gt; hoặc CRUD cho mọi bảng trước. Spring JDBC đã xử lý kết nối/statement/exception; chỉ trích helper khi có nhu cầu thực tế.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="72" customHeight="1">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giới hạn cách chia</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model trong cùng thư mục không đồng nghĩa cả nhóm được ghi mọi bảng. Owner giữ quy tắc ghi; các consumer dùng projection/cổng đọc đã bàn giao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="72" customHeight="1">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giới hạn cách chia</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không giao A viết toàn bộ model, B toàn bộ repository, C toàn bộ service. Mỗi owner hoàn thiện phần dữ liệu và luồng của chức năng mình; A giữ hạ tầng chung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="72" customHeight="1">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giới hạn cách chia</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Các tên file/hàm ở đây là đề xuất cần chốt tại task, chưa phải API Java đã tồn tại. Các mục này không tạo thêm task, đổi STT hay tự đánh dấu tiến độ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="72" customHeight="1">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring JDBC: RowMapper có thể tái sử dụng</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/docs/6.2.x/javadoc-api/org/springframework/jdbc/core/RowMapper.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="72" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring: transaction tại service và cơ chế proxy</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/reference/6.2/data-access/transaction/declarative/annotations.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="72" customHeight="1">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martin Fowler: chi phí xây dựng trước nhu cầu (Yagni)</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://martinfowler.com/bliki/Yagni.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="72" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Main class và package</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đặt TrodayApplication trong com.troday; package ngay bên dưới là controller, service, repository, model, dto, config, security, exception, integration, util. Các chức năng dùng chung các tầng này, phân biệt bằng tên lớp; không tạo lại cây package theo chức năng hoặc A/B/C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="72" customHeight="1">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bean và route theo tầng</t>
+        </is>
+      </c>
+      <c r="B103" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controller dùng @RestController/@RequestMapping, nghiệp vụ @Service, truy cập SQL @Repository; constructor injection. Các route của từng chức năng nằm trong controller tương ứng, Spring quét bean dưới com.troday.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="72" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DTO, kiểu số và ngày</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Request/response DTO nằm trong dto/request và dto/response, có @Valid và Bean Validation. Tiền dùng BigDecimal; ID JSON giữ chuỗi; Instant cho UTC, LocalDate cho ngày Việt Nam. ApiResponse/PageMeta trong dto/response; lỗi trong exception; ActorContext trong security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="72" customHeight="1">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giao dịch do service quản lý</t>
+        </is>
+      </c>
+      <c r="B105" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dùng @Transactional tại service public hoặc TransactionTemplate cho thao tác tự ghi nhiều bảng. Các repository/cổng đọc dùng cùng DataSource và transaction Spring; không commit riêng trong implementation. Tham số tx là ngữ cảnh server, không truyền JDBC Connection qua HTTP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="72" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giao dịch do procedure quản lý</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">StoredProcedureGateway nằm trong repository/procedure, là bean riêng gọi SimpleJdbcCall/CallableStatement với IN/OUT tường minh. Dùng Propagation.NEVER khi CALL tự START/COMMIT; không self-invocation bỏ qua guard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="72" customHeight="1">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tôn trọng SQL hiện có</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MySQL CHECK/FK/trigger và thủ tục giữ ràng buộc hiện có. Model trong model/ dùng Spring JDBC; không bật ORM tự tạo/cập nhật schema. Client kho tệp/email/push đặt trong integration/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="72" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Không tạo vòng phụ thuộc bean</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interface bàn giao đặt trong service/, implementation đọc SQL đặt trong repository/. Không inject ngược các service nghiệp vụ vào nhau hoặc dùng @Lazy để che vòng phụ thuộc. Event/audit/idempotency cũng dùng lớp trong service/repository; helper thời gian trong util/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="72" customHeight="1">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test và cấu hình dùng chung</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test lớp đặt vào package cùng tầng; test tích hợp/contract/e2e vào các thư mục theo loại kiểm thử. Fixture Java dùng support/fixtures, SQL dùng src/test/resources/sql; đặt tên theo chức năng, không chia thư mục A/B/C. A giữ build, main class, config và profile; mỗi người giữ các lớp nghiệp vụ của mình xuyên các tầng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="72" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Đường dẫn và quyền sửa file</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BE/... tính từ root repository troday. database/source và scripts/build-database.cjs trong kế hoạch là nguồn SQL/công cụ của wireframe hiện tại; A tích hợp output vào troday/database. {House,Room} biểu thị các tên lớp thay thế; * biểu thị phần tên theo task. Phân công theo chức năng và tên lớp, không dành cả một tầng cho một người.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="72" customHeight="1">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chạy local</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd spring-boot:run "-Dspring-boot.run.profiles=local"
+Chạy trong troday/BE; cấu hình MySQL local và biến môi trường.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="72" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unit/controller tests</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd test
+Smoke test hiện có không truy cập MySQL; bổ sung test theo từng task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="72" customHeight="1">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiểm thử và đóng gói</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.\mvnw.cmd verify
+Hiện chạy smoke test và đóng gói JAR; test SQL cần MySQL test độc lập khi triển khai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="72" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Linux/macOS</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">./mvnw test
+Chạy ./mvnw verify để kiểm thử và đóng gói.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="72" customHeight="1">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring Boot: bố trí main class và package</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-boot/reference/using/structuring-your-code.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="72" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring JDBC: SimpleJdbcCall</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/reference/data-access/jdbc/simple.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="72" customHeight="1">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spring: Propagation.NEVER</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://docs.spring.io/spring-framework/docs/current/javadoc-api/org/springframework/transaction/annotation/Propagation.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="72" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Spring Boot: tương thích Java và build tools</t>
         </is>
       </c>
-      <c r="B94" s="2" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://docs.spring.io/spring-boot/system-requirements.html</t>
         </is>
@@ -2187,12 +2635,12 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ngày kế hoạch</t>
+          <t xml:space="preserve">Ngày cập nhật</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-29</t>
+          <t xml:space="preserve">2026-10-31</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2753,7 +3201,7 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test module / DB</t>
+          <t xml:space="preserve">Test chức năng / DB</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -2864,27 +3312,35 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/src/main/resources/application*.yml
-backend/src/test/resources/application-test.yml
-backend/src/test/java/com/troday/e2e/release/**</t>
+BE/src/main/resources/application*.yml
+BE/src/test/resources/application-test.yml
+BE/src/test/java/com/troday/e2e/ReleaseE2ETests.java</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2904,8 +3360,8 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tạo backend/pom.xml, Maven Wrapper, TrodayApplication trong com.troday, package chức năng và resources profiles; Spring component scan nhận bean.
-Chọn starters Web MVC/Validation/Security/JDBC, MySQL driver và test tương thích; CI chạy Maven test/verify trên DB test riêng.
+          <t xml:space="preserve">Rà soát BE/pom.xml, Maven Wrapper, TrodayApplication trong com.troday, các tầng controller/service/repository/model/dto và resources profiles; Spring component scan nhận bean.
+Kiểm tra starters Web MVC/Validation/Security/JDBC, MySQL driver và test tương thích; CI chạy Maven test/verify trên DB test riêng.
 CI dựng SQL nguồn vào thư mục tạm, không bật ORM tự tạo/cập nhật schema; nhánh be/&lt;owner&gt;/&lt;task-id&gt;-&lt;slug&gt; và review bắt buộc.</t>
         </is>
       </c>
@@ -3029,7 +3485,7 @@
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chốt module nhà/tin/lịch và dữ liệu bàn giao</t>
+          <t xml:space="preserve">Chốt chức năng nhà/tin/lịch và dữ liệu bàn giao</t>
         </is>
       </c>
       <c r="G3" s="0">
@@ -3045,29 +3501,80 @@
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**
-backend/src/main/java/com/troday/posts/**
-backend/src/test/java/com/troday/posts/**
-backend/docs/contracts/posts.json
-backend/src/main/java/com/troday/services/**
-backend/src/test/java/com/troday/services/**
-backend/docs/contracts/services.json
-backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**
-backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java
+BE/src/main/java/com/troday/controller/{Post,PublicPost,Favorite}Controller.java
+BE/src/main/java/com/troday/service/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/mapper/{Post,PublicPost,Favorite}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Post,PublicPost,Favorite}*Gateway.java
+BE/src/main/java/com/troday/model/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/dto/request/*{Post,PublicPost,Favorite}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Post,PublicPost,Favorite}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Post,PublicPost,Favorite}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Post,PublicPost,Favorite}*Fixtures.java
+BE/src/test/resources/sql/{post,public-post,favorite}-*.sql
+BE/docs/contracts/*{post,public-post,favorite}*.json
+BE/src/main/java/com/troday/controller/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}Controller.java
+BE/src/main/java/com/troday/service/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/mapper/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Gateway.java
+BE/src/main/java/com/troday/model/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/dto/request/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Request.java
+BE/src/main/java/com/troday/dto/response/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Fixtures.java
+BE/src/test/resources/sql/{rental-service,house-rental-service,room-rental-service,service-quote}-*.sql
+BE/docs/contracts/*{rental-service,house-rental-service,room-rental-service,service-quote}*.json
+BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java
+BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K3" s="0" t="inlineStr">
@@ -3088,7 +3595,7 @@
       <c r="N3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Phân biệt postId/roomId, quyền nhà, capacity load, quote service và trạng thái kết nối.
-Tạo fixture trong backend/src/test/java/com/troday/support/fixtures/b/**; không sửa seed chung của A/C.
+Tạo BE/src/test/java/com/troday/support/fixtures/PropertyFixtures.java và SQL fixture property-*.sql trong BE/src/test/resources/sql; không sửa fixture của chức năng A/C.
 Gửi đề xuất IF-ROOM/IF-SERVICE/IF-CONNECTION để C01 phân tích thuê và A02 chốt contract v1 ở các lượt tiếp theo.</t>
         </is>
       </c>
@@ -3228,16 +3735,22 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -3398,20 +3911,28 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml</t>
         </is>
       </c>
@@ -3432,8 +3953,8 @@
       </c>
       <c r="N5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Công bố backend/docs/contracts/core.json cùng Java record ActorContext/ApiResponse, DTO validation và error mapping trong shared/.
-Service tự ghi dùng @Transactional/TransactionTemplate; StoredProcedureGateway là bean riêng dùng Propagation.NEVER khi CALL tự START/COMMIT; actor lấy từ SecurityContext.
+          <t xml:space="preserve">Công bố BE/docs/contracts/core.json; ActorContext đặt trong security, ApiResponse trong dto/response, validation trong dto/request, xử lý lỗi trong exception.
+Service tự ghi dùng @Transactional/TransactionTemplate; StoredProcedureGateway trong repository/procedure là bean riêng dùng Propagation.NEVER khi CALL tự START/COMMIT; actor lấy từ SecurityContext.
 Định nghĩa eventId/recipient/eventKey, idempotency scope, whitelist audit target; constructor injection và contract test JUnit sẵn cho B/C.</t>
         </is>
       </c>
@@ -3573,9 +4094,18 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
-backend/src/test/java/com/troday/identity/**
-backend/docs/contracts/identity.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}Controller.java
+BE/src/main/java/com/troday/service/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/mapper/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Gateway.java
+BE/src/main/java/com/troday/model/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/dto/request/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Request.java
+BE/src/main/java/com/troday/dto/response/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Fixtures.java
+BE/src/test/resources/sql/{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}-*.sql
+BE/docs/contracts/*{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}*.json</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -3602,7 +4132,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thiếu token 401; sai scope/LOCKED không truy cập được tài nguyên module khác.
+          <t xml:space="preserve">Thiếu token 401; sai scope/LOCKED không truy cập được tài nguyên chức năng khác.
 Mọi contact/ID/money/date validate theo đặc tả, không log secret.</t>
         </is>
       </c>
@@ -3736,27 +4266,35 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/src/main/resources/application*.yml
-backend/src/test/resources/application-test.yml
-backend/src/test/java/com/troday/e2e/release/**</t>
+BE/src/main/resources/application*.yml
+BE/src/test/resources/application-test.yml
+BE/src/test/java/com/troday/e2e/ReleaseE2ETests.java</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
@@ -3917,9 +4455,20 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/files/**
-backend/src/test/java/com/troday/files/**
-backend/docs/contracts/files.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/FileController.java
+BE/src/main/java/com/troday/service/File*.java
+BE/src/main/java/com/troday/repository/File*.java
+BE/src/main/java/com/troday/repository/mapper/FileRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/File*Gateway.java
+BE/src/main/java/com/troday/model/File*.java
+BE/src/main/java/com/troday/dto/request/*File*Request.java
+BE/src/main/java/com/troday/dto/response/*File*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/File*Tests.java
+BE/src/test/java/com/troday/support/fixtures/File*Fixtures.java
+BE/src/test/resources/sql/file-*.sql
+BE/docs/contracts/*file*.json
+BE/src/main/java/com/troday/integration/FileStorage*.java
+BE/src/test/java/com/troday/integration/FileStorage*Tests.java</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -4080,9 +4629,18 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
-backend/src/test/java/com/troday/identity/**
-backend/docs/contracts/identity.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}Controller.java
+BE/src/main/java/com/troday/service/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/mapper/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Gateway.java
+BE/src/main/java/com/troday/model/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/dto/request/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Request.java
+BE/src/main/java/com/troday/dto/response/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Fixtures.java
+BE/src/test/resources/sql/{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}-*.sql
+BE/docs/contracts/*{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}*.json</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
@@ -4243,9 +4801,18 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
-backend/src/test/java/com/troday/identity/**
-backend/docs/contracts/identity.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}Controller.java
+BE/src/main/java/com/troday/service/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/mapper/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Gateway.java
+BE/src/main/java/com/troday/model/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/dto/request/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Request.java
+BE/src/main/java/com/troday/dto/response/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Fixtures.java
+BE/src/test/resources/sql/{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}-*.sql
+BE/docs/contracts/*{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}*.json</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -4406,16 +4973,31 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java</t>
         </is>
       </c>
       <c r="K11" s="0" t="inlineStr">
@@ -4576,9 +5158,18 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/services/**
-backend/src/test/java/com/troday/services/**
-backend/docs/contracts/services.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}Controller.java
+BE/src/main/java/com/troday/service/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/mapper/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Gateway.java
+BE/src/main/java/com/troday/model/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/dto/request/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Request.java
+BE/src/main/java/com/troday/dto/response/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Fixtures.java
+BE/src/test/resources/sql/{rental-service,house-rental-service,room-rental-service,service-quote}-*.sql
+BE/docs/contracts/*{rental-service,house-rental-service,room-rental-service,service-quote}*.json</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -4739,22 +5330,55 @@
       </c>
       <c r="J13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**
-backend/src/main/java/com/troday/services/**
-backend/src/test/java/com/troday/services/**
-backend/docs/contracts/services.json
-backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java
+BE/src/main/java/com/troday/controller/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}Controller.java
+BE/src/main/java/com/troday/service/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/mapper/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Gateway.java
+BE/src/main/java/com/troday/model/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/dto/request/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Request.java
+BE/src/main/java/com/troday/dto/response/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Fixtures.java
+BE/src/test/resources/sql/{rental-service,house-rental-service,room-rental-service,service-quote}-*.sql
+BE/docs/contracts/*{rental-service,house-rental-service,room-rental-service,service-quote}*.json
+BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
@@ -4915,13 +5539,19 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -5082,13 +5712,19 @@
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
@@ -5249,20 +5885,35 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -5423,13 +6074,22 @@
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
-backend/src/test/java/com/troday/posts/**
-backend/docs/contracts/posts.json
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Post,PublicPost,Favorite}Controller.java
+BE/src/main/java/com/troday/service/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/mapper/{Post,PublicPost,Favorite}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Post,PublicPost,Favorite}*Gateway.java
+BE/src/main/java/com/troday/model/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/dto/request/*{Post,PublicPost,Favorite}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Post,PublicPost,Favorite}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Post,PublicPost,Favorite}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Post,PublicPost,Favorite}*Fixtures.java
+BE/src/test/resources/sql/{post,public-post,favorite}-*.sql
+BE/docs/contracts/*{post,public-post,favorite}*.json
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
@@ -5451,7 +6111,7 @@
         <is>
           <t xml:space="preserve">sp_submit_post nhận/ghi ảnh+amenities cùng transaction, content_version và quota 3 slot đúng hiện tại.
 Edit giữ roomId; pending edit không chiếm thêm lượt; moderate/hide/restore theo đúng postId.
-Các /admin/posts ở module posts; không sửa account-admin controller của A.</t>
+Các /admin/posts nằm trong controller/PostController.java của B; không sửa AccountAdminController của A.</t>
         </is>
       </c>
       <c r="O17" s="0" t="inlineStr">
@@ -5590,19 +6250,43 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
-backend/src/test/java/com/troday/posts/**
-backend/docs/contracts/posts.json
-backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Post,PublicPost,Favorite}Controller.java
+BE/src/main/java/com/troday/service/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/mapper/{Post,PublicPost,Favorite}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Post,PublicPost,Favorite}*Gateway.java
+BE/src/main/java/com/troday/model/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/dto/request/*{Post,PublicPost,Favorite}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Post,PublicPost,Favorite}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Post,PublicPost,Favorite}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Post,PublicPost,Favorite}*Fixtures.java
+BE/src/test/resources/sql/{post,public-post,favorite}-*.sql
+BE/docs/contracts/*{post,public-post,favorite}*.json
+BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -5763,16 +6447,22 @@
       </c>
       <c r="J19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K19" s="0" t="inlineStr">
@@ -5933,12 +6623,30 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -6099,12 +6807,30 @@
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
@@ -6265,14 +6991,23 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -6433,14 +7168,23 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
@@ -6601,16 +7345,22 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -6771,10 +7521,19 @@
       </c>
       <c r="J25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java</t>
         </is>
       </c>
       <c r="K25" s="0" t="inlineStr">
@@ -6935,16 +7694,22 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -7105,16 +7870,22 @@
       </c>
       <c r="J27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K27" s="0" t="inlineStr">
@@ -7275,13 +8046,19 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -7442,9 +8219,18 @@
       </c>
       <c r="J29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K29" s="0" t="inlineStr">
@@ -7605,9 +8391,18 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -7768,9 +8563,18 @@
       </c>
       <c r="J31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K31" s="0" t="inlineStr">
@@ -7931,12 +8735,30 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -8097,13 +8919,19 @@
       </c>
       <c r="J33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="K33" s="0" t="inlineStr">
@@ -8264,9 +9092,18 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
-backend/src/test/java/com/troday/billing/**
-backend/docs/contracts/billing.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Invoice,Billing}Controller.java
+BE/src/main/java/com/troday/service/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/mapper/{Invoice,Billing}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Invoice,Billing}*Gateway.java
+BE/src/main/java/com/troday/model/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/dto/request/*{Invoice,Billing}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Invoice,Billing}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Invoice,Billing}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Invoice,Billing}*Fixtures.java
+BE/src/test/resources/sql/{invoice,billing}-*.sql
+BE/docs/contracts/*{invoice,billing}*.json</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -8427,15 +9264,42 @@
       </c>
       <c r="J35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/accountadmin/**
-backend/src/test/java/com/troday/accountadmin/**
-backend/src/main/java/com/troday/audit/**
-backend/src/test/java/com/troday/audit/**
-backend/src/main/java/com/troday/admindashboard/**
-backend/src/test/java/com/troday/admindashboard/**
-backend/docs/contracts/accountadmin.json
-backend/docs/contracts/audit.json
-backend/docs/contracts/admindashboard.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/AccountAdminController.java
+BE/src/main/java/com/troday/service/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/mapper/AccountAdminRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AccountAdmin*Gateway.java
+BE/src/main/java/com/troday/model/AccountAdmin*.java
+BE/src/main/java/com/troday/dto/request/*AccountAdmin*Request.java
+BE/src/main/java/com/troday/dto/response/*AccountAdmin*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AccountAdmin*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AccountAdmin*Fixtures.java
+BE/src/test/resources/sql/account-admin-*.sql
+BE/docs/contracts/*account-admin*.json
+BE/src/main/java/com/troday/controller/AuditController.java
+BE/src/main/java/com/troday/service/Audit*.java
+BE/src/main/java/com/troday/repository/Audit*.java
+BE/src/main/java/com/troday/repository/mapper/AuditRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Audit*Gateway.java
+BE/src/main/java/com/troday/model/Audit*.java
+BE/src/main/java/com/troday/dto/request/*Audit*Request.java
+BE/src/main/java/com/troday/dto/response/*Audit*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Audit*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Audit*Fixtures.java
+BE/src/test/resources/sql/audit-*.sql
+BE/docs/contracts/*audit*.json
+BE/src/main/java/com/troday/controller/AdminDashboardController.java
+BE/src/main/java/com/troday/service/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/mapper/AdminDashboardRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AdminDashboard*Gateway.java
+BE/src/main/java/com/troday/model/AdminDashboard*.java
+BE/src/main/java/com/troday/dto/request/*AdminDashboard*Request.java
+BE/src/main/java/com/troday/dto/response/*AdminDashboard*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AdminDashboard*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AdminDashboard*Fixtures.java
+BE/src/test/resources/sql/admin-dashboard-*.sql
+BE/docs/contracts/*admin-dashboard*.json</t>
         </is>
       </c>
       <c r="K35" s="0" t="inlineStr">
@@ -8462,7 +9326,7 @@
       </c>
       <c r="O35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tài khoản bị khóa mất quyền trên mọi module qua cùng middleware.
+          <t xml:space="preserve">Tài khoản bị khóa mất quyền trên mọi chức năng qua cùng middleware.
 Khóa landlord làm public view mất quyền, nhưng hợp đồng/người ở cũ được giữ.</t>
         </is>
       </c>
@@ -8596,9 +9460,18 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
-backend/src/test/java/com/troday/billing/**
-backend/docs/contracts/billing.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Invoice,Billing}Controller.java
+BE/src/main/java/com/troday/service/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/mapper/{Invoice,Billing}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Invoice,Billing}*Gateway.java
+BE/src/main/java/com/troday/model/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/dto/request/*{Invoice,Billing}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Invoice,Billing}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Invoice,Billing}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Invoice,Billing}*Fixtures.java
+BE/src/test/resources/sql/{invoice,billing}-*.sql
+BE/docs/contracts/*{invoice,billing}*.json</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -8759,16 +9632,22 @@
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
@@ -8929,16 +9808,22 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -9099,16 +9984,22 @@
       </c>
       <c r="J39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K39" s="0" t="inlineStr">
@@ -9269,12 +10160,30 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -9435,12 +10344,30 @@
       </c>
       <c r="J41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
-backend/src/test/java/com/troday/reviews/**
-backend/src/main/java/com/troday/reports/**
-backend/src/test/java/com/troday/reports/**
-backend/docs/contracts/reviews.json
-backend/docs/contracts/reports.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/ReviewController.java
+BE/src/main/java/com/troday/service/Review*.java
+BE/src/main/java/com/troday/repository/Review*.java
+BE/src/main/java/com/troday/repository/mapper/ReviewRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Review*Gateway.java
+BE/src/main/java/com/troday/model/Review*.java
+BE/src/main/java/com/troday/dto/request/*Review*Request.java
+BE/src/main/java/com/troday/dto/response/*Review*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Review*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Review*Fixtures.java
+BE/src/test/resources/sql/review-*.sql
+BE/docs/contracts/*review*.json
+BE/src/main/java/com/troday/controller/ReportController.java
+BE/src/main/java/com/troday/service/Report*.java
+BE/src/main/java/com/troday/repository/Report*.java
+BE/src/main/java/com/troday/repository/mapper/ReportRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Report*Gateway.java
+BE/src/main/java/com/troday/model/Report*.java
+BE/src/main/java/com/troday/dto/request/*Report*Request.java
+BE/src/main/java/com/troday/dto/response/*Report*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Report*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Report*Fixtures.java
+BE/src/test/resources/sql/report-*.sql
+BE/docs/contracts/*report*.json</t>
         </is>
       </c>
       <c r="K41" s="0" t="inlineStr">
@@ -9601,36 +10528,71 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml
-backend/src/main/java/com/troday/accountadmin/**
-backend/src/test/java/com/troday/accountadmin/**
-backend/src/main/java/com/troday/audit/**
-backend/src/test/java/com/troday/audit/**
-backend/src/main/java/com/troday/admindashboard/**
-backend/src/test/java/com/troday/admindashboard/**
-backend/docs/contracts/accountadmin.json
-backend/docs/contracts/audit.json
-backend/docs/contracts/admindashboard.json
+BE/src/main/java/com/troday/controller/AccountAdminController.java
+BE/src/main/java/com/troday/service/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/mapper/AccountAdminRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AccountAdmin*Gateway.java
+BE/src/main/java/com/troday/model/AccountAdmin*.java
+BE/src/main/java/com/troday/dto/request/*AccountAdmin*Request.java
+BE/src/main/java/com/troday/dto/response/*AccountAdmin*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AccountAdmin*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AccountAdmin*Fixtures.java
+BE/src/test/resources/sql/account-admin-*.sql
+BE/docs/contracts/*account-admin*.json
+BE/src/main/java/com/troday/controller/AuditController.java
+BE/src/main/java/com/troday/service/Audit*.java
+BE/src/main/java/com/troday/repository/Audit*.java
+BE/src/main/java/com/troday/repository/mapper/AuditRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Audit*Gateway.java
+BE/src/main/java/com/troday/model/Audit*.java
+BE/src/main/java/com/troday/dto/request/*Audit*Request.java
+BE/src/main/java/com/troday/dto/response/*Audit*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Audit*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Audit*Fixtures.java
+BE/src/test/resources/sql/audit-*.sql
+BE/docs/contracts/*audit*.json
+BE/src/main/java/com/troday/controller/AdminDashboardController.java
+BE/src/main/java/com/troday/service/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/mapper/AdminDashboardRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AdminDashboard*Gateway.java
+BE/src/main/java/com/troday/model/AdminDashboard*.java
+BE/src/main/java/com/troday/dto/request/*AdminDashboard*Request.java
+BE/src/main/java/com/troday/dto/response/*AdminDashboard*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AdminDashboard*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AdminDashboard*Fixtures.java
+BE/src/test/resources/sql/admin-dashboard-*.sql
+BE/docs/contracts/*admin-dashboard*.json
 database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/src/main/resources/application*.yml
-backend/src/test/resources/application-test.yml
-backend/src/test/java/com/troday/e2e/release/**</t>
+BE/src/main/resources/application*.yml
+BE/src/test/resources/application-test.yml
+BE/src/test/java/com/troday/e2e/ReleaseE2ETests.java</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -9791,9 +10753,18 @@
       </c>
       <c r="J43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="K43" s="0" t="inlineStr">
@@ -9954,12 +10925,30 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
-backend/src/test/java/com/troday/reviews/**
-backend/src/main/java/com/troday/reports/**
-backend/src/test/java/com/troday/reports/**
-backend/docs/contracts/reviews.json
-backend/docs/contracts/reports.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/ReviewController.java
+BE/src/main/java/com/troday/service/Review*.java
+BE/src/main/java/com/troday/repository/Review*.java
+BE/src/main/java/com/troday/repository/mapper/ReviewRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Review*Gateway.java
+BE/src/main/java/com/troday/model/Review*.java
+BE/src/main/java/com/troday/dto/request/*Review*Request.java
+BE/src/main/java/com/troday/dto/response/*Review*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Review*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Review*Fixtures.java
+BE/src/test/resources/sql/review-*.sql
+BE/docs/contracts/*review*.json
+BE/src/main/java/com/troday/controller/ReportController.java
+BE/src/main/java/com/troday/service/Report*.java
+BE/src/main/java/com/troday/repository/Report*.java
+BE/src/main/java/com/troday/repository/mapper/ReportRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Report*Gateway.java
+BE/src/main/java/com/troday/model/Report*.java
+BE/src/main/java/com/troday/dto/request/*Report*Request.java
+BE/src/main/java/com/troday/dto/response/*Report*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Report*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Report*Fixtures.java
+BE/src/test/resources/sql/report-*.sql
+BE/docs/contracts/*report*.json</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -10120,16 +11109,31 @@
       </c>
       <c r="J45" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java</t>
         </is>
       </c>
       <c r="K45" s="0" t="inlineStr">
@@ -10150,7 +11154,7 @@
       <c r="N45" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Scope landlord cho từng metric; ACTIVE tính occupied, không đồng nhất reserved với occupied.
-Lịch chưa hết giờ, hóa đơn UNPAID/OVERDUE và pending requests có nguồn đúng module.
+Lịch chưa hết giờ, hóa đơn UNPAID/OVERDUE và pending requests có nguồn đúng chức năng.
 Có asOf, tách truy vấn count khỏi trả danh tính cư dân.</t>
         </is>
       </c>
@@ -10290,20 +11294,35 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java
 database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -10464,16 +11483,22 @@
       </c>
       <c r="J47" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K47" s="0" t="inlineStr">
@@ -10634,16 +11659,22 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -10804,16 +11835,22 @@
       </c>
       <c r="J49" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java
 database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="K49" s="0" t="inlineStr">
@@ -10958,7 +11995,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm thử module nhà/tin/lịch và nội dung</t>
+          <t xml:space="preserve">Kiểm thử chức năng nhà/tin/lịch và nội dung</t>
         </is>
       </c>
       <c r="G50" s="2">
@@ -10974,32 +12011,92 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**
-backend/src/main/java/com/troday/posts/**
-backend/src/test/java/com/troday/posts/**
-backend/docs/contracts/posts.json
-backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**
-backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json
-backend/src/main/java/com/troday/reviews/**
-backend/src/test/java/com/troday/reviews/**
-backend/src/main/java/com/troday/reports/**
-backend/src/test/java/com/troday/reports/**
-backend/docs/contracts/reviews.json
-backend/docs/contracts/reports.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java
+BE/src/main/java/com/troday/controller/{Post,PublicPost,Favorite}Controller.java
+BE/src/main/java/com/troday/service/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/mapper/{Post,PublicPost,Favorite}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Post,PublicPost,Favorite}*Gateway.java
+BE/src/main/java/com/troday/model/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/dto/request/*{Post,PublicPost,Favorite}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Post,PublicPost,Favorite}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Post,PublicPost,Favorite}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Post,PublicPost,Favorite}*Fixtures.java
+BE/src/test/resources/sql/{post,public-post,favorite}-*.sql
+BE/docs/contracts/*{post,public-post,favorite}*.json
+BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java
+BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json
+BE/src/main/java/com/troday/controller/ReviewController.java
+BE/src/main/java/com/troday/service/Review*.java
+BE/src/main/java/com/troday/repository/Review*.java
+BE/src/main/java/com/troday/repository/mapper/ReviewRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Review*Gateway.java
+BE/src/main/java/com/troday/model/Review*.java
+BE/src/main/java/com/troday/dto/request/*Review*Request.java
+BE/src/main/java/com/troday/dto/response/*Review*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Review*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Review*Fixtures.java
+BE/src/test/resources/sql/review-*.sql
+BE/docs/contracts/*review*.json
+BE/src/main/java/com/troday/controller/ReportController.java
+BE/src/main/java/com/troday/service/Report*.java
+BE/src/main/java/com/troday/repository/Report*.java
+BE/src/main/java/com/troday/repository/mapper/ReportRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Report*Gateway.java
+BE/src/main/java/com/troday/model/Report*.java
+BE/src/main/java/com/troday/dto/request/*Report*Request.java
+BE/src/main/java/com/troday/dto/response/*Report*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Report*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Report*Fixtures.java
+BE/src/test/resources/sql/report-*.sql
+BE/docs/contracts/*report*.json</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -11160,30 +12257,65 @@
       </c>
       <c r="J51" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml
-backend/src/main/java/com/troday/billing/**
-backend/src/test/java/com/troday/billing/**
-backend/docs/contracts/billing.json
-backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+BE/src/main/java/com/troday/controller/{Invoice,Billing}Controller.java
+BE/src/main/java/com/troday/service/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/mapper/{Invoice,Billing}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Invoice,Billing}*Gateway.java
+BE/src/main/java/com/troday/model/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/dto/request/*{Invoice,Billing}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Invoice,Billing}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Invoice,Billing}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Invoice,Billing}*Fixtures.java
+BE/src/test/resources/sql/{invoice,billing}-*.sql
+BE/docs/contracts/*{invoice,billing}*.json
+BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="K51" s="0" t="inlineStr">
@@ -11328,7 +12460,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">E2E thuê xuyên ba module và bàn giao API</t>
+          <t xml:space="preserve">E2E thuê xuyên các chức năng và bàn giao API</t>
         </is>
       </c>
       <c r="G52" s="2">
@@ -11344,13 +12476,19 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -11514,9 +12652,9 @@
           <t xml:space="preserve">database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/src/main/resources/application*.yml
-backend/src/test/resources/application-test.yml
-backend/src/test/java/com/troday/e2e/release/**</t>
+BE/src/main/resources/application*.yml
+BE/src/test/resources/application-test.yml
+BE/src/test/java/com/troday/e2e/ReleaseE2ETests.java</t>
         </is>
       </c>
       <c r="K53" s="0" t="inlineStr">
@@ -11537,7 +12675,7 @@
       <c r="N53" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">Tái sinh schema từ toàn bộ source, chốt thứ tự migration; test tạo mới/nâng cấp trên DB tạm.
-Đối chiếu 176 API có đúng một task/module owner, gom collection/API docs và hướng dẫn chạy.
+Đối chiếu 176 API có đúng một task và người phụ trách, gom collection/API docs và hướng dẫn chạy.
 Xác nhận G0–G6 và report E2E C16 trước bàn giao; chốt G7 sau khi A17 hoàn thành, không dùng gate chứa chính A17 làm điều kiện bắt đầu.</t>
         </is>
       </c>
@@ -24154,7 +25292,7 @@
     <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Module</t>
+          <t xml:space="preserve">Chức năng</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -24191,31 +25329,39 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/shared/**
-backend/src/main/java/com/troday/config/**
-backend/src/main/java/com/troday/TrodayApplication.java
-backend/src/test/java/com/troday/shared/**
-backend/src/test/java/com/troday/config/**
-backend/src/test/java/com/troday/support/fixtures/a/**
-backend/src/test/java/com/troday/contract/a/**
-backend/src/test/java/com/troday/e2e/platform/**
-backend/src/test/resources/sql/a/**
-backend/docs/contracts/core.json
-backend/pom.xml
-backend/mvnw
-backend/mvnw.cmd
-backend/.mvn/**
+          <t xml:space="preserve">BE/src/main/java/com/troday/config/**
+BE/src/main/java/com/troday/security/**
+BE/src/main/java/com/troday/exception/**
+BE/src/main/java/com/troday/util/**
+BE/src/main/java/com/troday/dto/request/PageQuery.java
+BE/src/main/java/com/troday/dto/response/{ApiResponse,PageMeta}.java
+BE/src/main/java/com/troday/service/{Idempotency,Event,Audit}*.java
+BE/src/main/java/com/troday/repository/{Idempotency,Event}*.java
+BE/src/main/java/com/troday/repository/procedure/StoredProcedureGateway.java
+BE/src/main/java/com/troday/TrodayApplication.java
+BE/src/test/java/com/troday/{config,security,exception}/**
+BE/src/test/java/com/troday/service/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/repository/{Idempotency,Event}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/PlatformFixtures.java
+BE/src/test/java/com/troday/contract/CoreContractTests.java
+BE/src/test/java/com/troday/e2e/PlatformE2ETests.java
+BE/src/test/resources/sql/platform-*.sql
+BE/docs/contracts/core*.json
+BE/pom.xml
+BE/mvnw
+BE/mvnw.cmd
+BE/.mvn/**
 .github/workflows/backend.yml</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ActorContext, ApiResponse, Spring Security/config, transaction/procedure gateway, idempotency và event/audit ports.</t>
+          <t xml:space="preserve">ActorContext trong security; ApiResponse trong dto/response; lỗi trong exception; gateway trong repository/procedure; event/audit/idempotency trong service/repository.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A giữ main class/config/POM. B/C thêm bean trong package chức năng, Spring component scan nhận tự động; không có manifest hoặc routes.* chung.</t>
+          <t xml:space="preserve">A giữ main class/config/POM và lớp dùng chung. B/C thêm lớp nghiệp vụ vào các tầng controller/service/repository/model/dto, Spring component scan nhận tự động.</t>
         </is>
       </c>
     </row>
@@ -24232,9 +25378,18 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/identity/**
-backend/src/test/java/com/troday/identity/**
-backend/docs/contracts/identity.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}Controller.java
+BE/src/main/java/com/troday/service/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/repository/mapper/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Gateway.java
+BE/src/main/java/com/troday/model/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*.java
+BE/src/main/java/com/troday/dto/request/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Request.java
+BE/src/main/java/com/troday/dto/response/*{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{User,AuthSession,Auth,Account,Profile,Session,Verification,PasswordReset,Token,Identity}*Fixtures.java
+BE/src/test/resources/sql/{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}-*.sql
+BE/docs/contracts/*{user,auth-session,auth,account,profile,session,verification,password-reset,token,identity}*.json</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -24261,9 +25416,20 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/files/**
-backend/src/test/java/com/troday/files/**
-backend/docs/contracts/files.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/FileController.java
+BE/src/main/java/com/troday/service/File*.java
+BE/src/main/java/com/troday/repository/File*.java
+BE/src/main/java/com/troday/repository/mapper/FileRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/File*Gateway.java
+BE/src/main/java/com/troday/model/File*.java
+BE/src/main/java/com/troday/dto/request/*File*Request.java
+BE/src/main/java/com/troday/dto/response/*File*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/File*Tests.java
+BE/src/test/java/com/troday/support/fixtures/File*Fixtures.java
+BE/src/test/resources/sql/file-*.sql
+BE/docs/contracts/*file*.json
+BE/src/main/java/com/troday/integration/FileStorage*.java
+BE/src/test/java/com/troday/integration/FileStorage*Tests.java</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -24290,12 +25456,30 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/messaging/**
-backend/src/test/java/com/troday/messaging/**
-backend/src/main/java/com/troday/notifications/**
-backend/src/test/java/com/troday/notifications/**
-backend/docs/contracts/messaging.json
-backend/docs/contracts/notifications.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Conversation,Message,Chat}Controller.java
+BE/src/main/java/com/troday/service/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/repository/mapper/{Conversation,Message,Chat}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Conversation,Message,Chat}*Gateway.java
+BE/src/main/java/com/troday/model/{Conversation,Message,Chat}*.java
+BE/src/main/java/com/troday/dto/request/*{Conversation,Message,Chat}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Conversation,Message,Chat}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Conversation,Message,Chat}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Conversation,Message,Chat}*Fixtures.java
+BE/src/test/resources/sql/{conversation,message,chat}-*.sql
+BE/docs/contracts/*{conversation,message,chat}*.json
+BE/src/main/java/com/troday/controller/{Notification,Sse}Controller.java
+BE/src/main/java/com/troday/service/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/{Notification,Sse}*.java
+BE/src/main/java/com/troday/repository/mapper/{Notification,Sse}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Notification,Sse}*Gateway.java
+BE/src/main/java/com/troday/model/{Notification,Sse}*.java
+BE/src/main/java/com/troday/dto/request/*{Notification,Sse}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Notification,Sse}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Notification,Sse}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Notification,Sse}*Fixtures.java
+BE/src/test/resources/sql/{notification,sse}-*.sql
+BE/docs/contracts/*{notification,sse}*.json</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
@@ -24322,9 +25506,18 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/billing/**
-backend/src/test/java/com/troday/billing/**
-backend/docs/contracts/billing.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Invoice,Billing}Controller.java
+BE/src/main/java/com/troday/service/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/repository/mapper/{Invoice,Billing}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Invoice,Billing}*Gateway.java
+BE/src/main/java/com/troday/model/{Invoice,Billing}*.java
+BE/src/main/java/com/troday/dto/request/*{Invoice,Billing}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Invoice,Billing}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Invoice,Billing}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Invoice,Billing}*Fixtures.java
+BE/src/test/resources/sql/{invoice,billing}-*.sql
+BE/docs/contracts/*{invoice,billing}*.json</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -24351,20 +25544,47 @@
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/accountadmin/**
-backend/src/test/java/com/troday/accountadmin/**
-backend/src/main/java/com/troday/audit/**
-backend/src/test/java/com/troday/audit/**
-backend/src/main/java/com/troday/admindashboard/**
-backend/src/test/java/com/troday/admindashboard/**
-backend/docs/contracts/accountadmin.json
-backend/docs/contracts/audit.json
-backend/docs/contracts/admindashboard.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/AccountAdminController.java
+BE/src/main/java/com/troday/service/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/AccountAdmin*.java
+BE/src/main/java/com/troday/repository/mapper/AccountAdminRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AccountAdmin*Gateway.java
+BE/src/main/java/com/troday/model/AccountAdmin*.java
+BE/src/main/java/com/troday/dto/request/*AccountAdmin*Request.java
+BE/src/main/java/com/troday/dto/response/*AccountAdmin*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AccountAdmin*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AccountAdmin*Fixtures.java
+BE/src/test/resources/sql/account-admin-*.sql
+BE/docs/contracts/*account-admin*.json
+BE/src/main/java/com/troday/controller/AuditController.java
+BE/src/main/java/com/troday/service/Audit*.java
+BE/src/main/java/com/troday/repository/Audit*.java
+BE/src/main/java/com/troday/repository/mapper/AuditRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Audit*Gateway.java
+BE/src/main/java/com/troday/model/Audit*.java
+BE/src/main/java/com/troday/dto/request/*Audit*Request.java
+BE/src/main/java/com/troday/dto/response/*Audit*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Audit*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Audit*Fixtures.java
+BE/src/test/resources/sql/audit-*.sql
+BE/docs/contracts/*audit*.json
+BE/src/main/java/com/troday/controller/AdminDashboardController.java
+BE/src/main/java/com/troday/service/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/AdminDashboard*.java
+BE/src/main/java/com/troday/repository/mapper/AdminDashboardRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/AdminDashboard*Gateway.java
+BE/src/main/java/com/troday/model/AdminDashboard*.java
+BE/src/main/java/com/troday/dto/request/*AdminDashboard*Request.java
+BE/src/main/java/com/troday/dto/response/*AdminDashboard*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/AdminDashboard*Tests.java
+BE/src/test/java/com/troday/support/fixtures/AdminDashboard*Fixtures.java
+BE/src/test/resources/sql/admin-dashboard-*.sql
+BE/docs/contracts/*admin-dashboard*.json</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Khóa phiên/tài khoản, truy vết và tổng quan quản trị; các /admin khác nằm tại package nghiệp vụ B/C.</t>
+          <t xml:space="preserve">Khóa phiên/tài khoản, truy vết và tổng quan quản trị; endpoint /admin của B/C đặt trong controller theo chức năng tương ứng.</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -24386,16 +25606,31 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/properties/**
-backend/src/test/java/com/troday/properties/**
-backend/src/main/java/com/troday/houserights/**
-backend/src/test/java/com/troday/houserights/**
-backend/docs/contracts/properties.json
-backend/docs/contracts/houserights.json
-backend/src/test/java/com/troday/support/fixtures/b/**
-backend/src/test/java/com/troday/contract/b/**
-backend/src/test/java/com/troday/e2e/property/**
-backend/src/test/resources/sql/b/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{House,Room,Property,LandlordDashboard}Controller.java
+BE/src/main/java/com/troday/service/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/repository/mapper/{House,Room,Property,LandlordDashboard}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{House,Room,Property,LandlordDashboard}*Gateway.java
+BE/src/main/java/com/troday/model/{House,Room,Property,LandlordDashboard}*.java
+BE/src/main/java/com/troday/dto/request/*{House,Room,Property,LandlordDashboard}*Request.java
+BE/src/main/java/com/troday/dto/response/*{House,Room,Property,LandlordDashboard}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{House,Room,Property,LandlordDashboard}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{House,Room,Property,LandlordDashboard}*Fixtures.java
+BE/src/test/resources/sql/{house,room,property,landlord-dashboard}-*.sql
+BE/docs/contracts/*{house,room,property,landlord-dashboard}*.json
+BE/src/main/java/com/troday/controller/HouseRightController.java
+BE/src/main/java/com/troday/service/HouseRight*.java
+BE/src/main/java/com/troday/repository/HouseRight*.java
+BE/src/main/java/com/troday/repository/mapper/HouseRightRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/HouseRight*Gateway.java
+BE/src/main/java/com/troday/model/HouseRight*.java
+BE/src/main/java/com/troday/dto/request/*HouseRight*Request.java
+BE/src/main/java/com/troday/dto/response/*HouseRight*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/HouseRight*Tests.java
+BE/src/test/java/com/troday/support/fixtures/HouseRight*Fixtures.java
+BE/src/test/resources/sql/house-right-*.sql
+BE/docs/contracts/*house-right*.json
+BE/src/test/java/com/troday/e2e/PropertyE2ETests.java</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -24405,7 +25640,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">C chỉ gọi Java port/SQL procedure dưới khóa; không đổi trạng thái phòng bằng setter từ controller.</t>
+          <t xml:space="preserve">C gọi interface trong service hoặc SQL procedure dưới khóa; không đổi trạng thái phòng bằng setter từ controller.</t>
         </is>
       </c>
     </row>
@@ -24422,9 +25657,18 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/posts/**
-backend/src/test/java/com/troday/posts/**
-backend/docs/contracts/posts.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Post,PublicPost,Favorite}Controller.java
+BE/src/main/java/com/troday/service/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/repository/mapper/{Post,PublicPost,Favorite}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Post,PublicPost,Favorite}*Gateway.java
+BE/src/main/java/com/troday/model/{Post,PublicPost,Favorite}*.java
+BE/src/main/java/com/troday/dto/request/*{Post,PublicPost,Favorite}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Post,PublicPost,Favorite}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Post,PublicPost,Favorite}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Post,PublicPost,Favorite}*Fixtures.java
+BE/src/test/resources/sql/{post,public-post,favorite}-*.sql
+BE/docs/contracts/*{post,public-post,favorite}*.json</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -24451,9 +25695,18 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/services/**
-backend/src/test/java/com/troday/services/**
-backend/docs/contracts/services.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}Controller.java
+BE/src/main/java/com/troday/service/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/repository/mapper/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Gateway.java
+BE/src/main/java/com/troday/model/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*.java
+BE/src/main/java/com/troday/dto/request/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Request.java
+BE/src/main/java/com/troday/dto/response/*{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{RentalService,HouseRentalService,RoomRentalService,ServiceQuote}*Fixtures.java
+BE/src/test/resources/sql/{rental-service,house-rental-service,room-rental-service,service-quote}-*.sql
+BE/docs/contracts/*{rental-service,house-rental-service,room-rental-service,service-quote}*.json</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -24480,10 +25733,19 @@
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/viewings/**
-backend/src/test/java/com/troday/viewings/**
-backend/docs/contracts/viewings.json
-backend/src/test/java/com/troday/e2e/viewingcontract/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Viewing,RentalDecision}Controller.java
+BE/src/main/java/com/troday/service/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/repository/mapper/{Viewing,RentalDecision}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Viewing,RentalDecision}*Gateway.java
+BE/src/main/java/com/troday/model/{Viewing,RentalDecision}*.java
+BE/src/main/java/com/troday/dto/request/*{Viewing,RentalDecision}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Viewing,RentalDecision}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Viewing,RentalDecision}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Viewing,RentalDecision}*Fixtures.java
+BE/src/test/resources/sql/{viewing,rental-decision}-*.sql
+BE/docs/contracts/*{viewing,rental-decision}*.json
+BE/src/test/java/com/troday/e2e/ViewingContractE2ETests.java</t>
         </is>
       </c>
       <c r="D11" s="0" t="inlineStr">
@@ -24510,9 +25772,18 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/roommates/**
-backend/src/test/java/com/troday/roommates/**
-backend/docs/contracts/roommates.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{Roommate,Connection,Matching,Criterion}Controller.java
+BE/src/main/java/com/troday/service/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/repository/mapper/{Roommate,Connection,Matching,Criterion}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{Roommate,Connection,Matching,Criterion}*Gateway.java
+BE/src/main/java/com/troday/model/{Roommate,Connection,Matching,Criterion}*.java
+BE/src/main/java/com/troday/dto/request/*{Roommate,Connection,Matching,Criterion}*Request.java
+BE/src/main/java/com/troday/dto/response/*{Roommate,Connection,Matching,Criterion}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{Roommate,Connection,Matching,Criterion}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{Roommate,Connection,Matching,Criterion}*Fixtures.java
+BE/src/test/resources/sql/{roommate,connection,matching,criterion}-*.sql
+BE/docs/contracts/*{roommate,connection,matching,criterion}*.json</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -24539,12 +25810,30 @@
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/reviews/**
-backend/src/test/java/com/troday/reviews/**
-backend/src/main/java/com/troday/reports/**
-backend/src/test/java/com/troday/reports/**
-backend/docs/contracts/reviews.json
-backend/docs/contracts/reports.json</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/ReviewController.java
+BE/src/main/java/com/troday/service/Review*.java
+BE/src/main/java/com/troday/repository/Review*.java
+BE/src/main/java/com/troday/repository/mapper/ReviewRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Review*Gateway.java
+BE/src/main/java/com/troday/model/Review*.java
+BE/src/main/java/com/troday/dto/request/*Review*Request.java
+BE/src/main/java/com/troday/dto/response/*Review*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Review*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Review*Fixtures.java
+BE/src/test/resources/sql/review-*.sql
+BE/docs/contracts/*review*.json
+BE/src/main/java/com/troday/controller/ReportController.java
+BE/src/main/java/com/troday/service/Report*.java
+BE/src/main/java/com/troday/repository/Report*.java
+BE/src/main/java/com/troday/repository/mapper/ReportRowMapper.java
+BE/src/main/java/com/troday/repository/procedure/Report*Gateway.java
+BE/src/main/java/com/troday/model/Report*.java
+BE/src/main/java/com/troday/dto/request/*Report*Request.java
+BE/src/main/java/com/troday/dto/response/*Report*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/Report*Tests.java
+BE/src/test/java/com/troday/support/fixtures/Report*Fixtures.java
+BE/src/test/resources/sql/report-*.sql
+BE/docs/contracts/*report*.json</t>
         </is>
       </c>
       <c r="D13" s="0" t="inlineStr">
@@ -24571,23 +25860,29 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/src/main/java/com/troday/rentals/**
-backend/src/test/java/com/troday/rentals/**
-backend/docs/contracts/rentals.json
-backend/src/test/java/com/troday/support/fixtures/c/**
-backend/src/test/java/com/troday/contract/c/**
-backend/src/test/java/com/troday/e2e/rental/**
-backend/src/test/resources/sql/c/**</t>
+          <t xml:space="preserve">BE/src/main/java/com/troday/controller/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}Controller.java
+BE/src/main/java/com/troday/service/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/repository/mapper/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}RowMapper.java
+BE/src/main/java/com/troday/repository/procedure/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Gateway.java
+BE/src/main/java/com/troday/model/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*.java
+BE/src/main/java/com/troday/dto/request/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Request.java
+BE/src/main/java/com/troday/dto/response/*{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Response.java
+BE/src/test/java/com/troday/{controller,service,repository,integration,contract}/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Tests.java
+BE/src/test/java/com/troday/support/fixtures/{ActiveStay,Contract,ContractRevision,ContractTemplate,Resident,Residency,OccupantJoin,RentalChange,Representative,Rental}*Fixtures.java
+BE/src/test/resources/sql/{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}-*.sql
+BE/docs/contracts/*{active-stay,contract,contract-revision,contract-template,resident,residency,occupant-join,rental-change,representative,rental}*.json
+BE/src/test/java/com/troday/e2e/RentalE2ETests.java</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contracts, revisions, room_tenants, history, join/change requests, templates và liên kết cư dân; tách package con.</t>
+          <t xml:space="preserve">Contracts, revisions, room_tenants, history, join/change requests, templates và liên kết cư dân; lớp đặt trực tiếp trong từng tầng.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Một transaction owner cho vào/rời/đổi phòng. Service Java dùng Spring transaction; CALL tự commit dùng gateway riêng.</t>
+          <t xml:space="preserve">Một transaction owner cho vào/rời/đổi phòng. Interface bàn giao nằm trong service; CALL tự commit dùng repository/procedure.</t>
         </is>
       </c>
     </row>
@@ -24607,7 +25902,7 @@
           <t xml:space="preserve">database/source/house-rights.sql
 database/source/post-review-quota.sql
 database/source/viewing-proposals.sql
-backend/src/test/java/com/troday/sqlproperty/**</t>
+BE/src/test/java/com/troday/integration/PropertySql*Tests.java</t>
         </is>
       </c>
       <c r="D15" s="0" t="inlineStr">
@@ -24636,7 +25931,7 @@
         <is>
           <t xml:space="preserve">database/source/workflows.sql
 database/source/contract-viewing-cleanup.sql
-backend/src/test/java/com/troday/sqlrental/**</t>
+BE/src/test/java/com/troday/integration/RentalSql*Tests.java</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -24666,9 +25961,9 @@
           <t xml:space="preserve">database/schema.sql
 database/migrations/*
 scripts/build-database.cjs
-backend/src/main/resources/application*.yml
-backend/src/test/resources/application-test.yml
-backend/src/test/java/com/troday/e2e/release/**</t>
+BE/src/main/resources/application*.yml
+BE/src/test/resources/application-test.yml
+BE/src/test/java/com/troday/e2e/ReleaseE2ETests.java</t>
         </is>
       </c>
       <c r="D17" s="0" t="inlineStr">
@@ -24798,7 +26093,7 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">A lần lượt hoàn tất auth, idempotency/audit, kho tệp, xét duyệt tài khoản và OTP/TokenPort. Các module sau nhận provider thật đã merge.</t>
+          <t xml:space="preserve">A lần lượt hoàn tất auth, idempotency/audit, kho tệp, xét duyệt tài khoản và OTP/TokenPort. Các chức năng sau nhận provider thật đã merge.</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
@@ -24816,7 +26111,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auth, audit mở rộng, idempotency, tệp, cấp vai trò và TokenPort đã chạy với DB/kho test, sẵn sàng cho module nghiệp vụ.</t>
+          <t xml:space="preserve">Auth, audit mở rộng, idempotency, tệp, cấp vai trò và TokenPort đã chạy với DB/kho test, sẵn sàng cho chức năng nghiệp vụ.</t>
         </is>
       </c>
       <c r="H3" s="0" t="str">
@@ -25032,7 +26327,7 @@
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">C kiểm thử giao dịch thuê, B kiểm thử module nhà/tin, A kiểm thử hạ tầng, C chạy E2E toàn hệ thống, cuối cùng A tích hợp bản release.</t>
+          <t xml:space="preserve">C kiểm thử giao dịch thuê, B kiểm thử chức năng nhà/tin, A kiểm thử hạ tầng, C chạy E2E toàn hệ thống, cuối cùng A tích hợp bản release.</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
@@ -25237,7 +26532,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Context resolver đăng ký theo module; proof đã nộp bất biến, không tạo import vòng.</t>
+          <t xml:space="preserve">Context resolver theo chức năng, lớp nằm trong service; proof đã nộp bất biến, không tạo import vòng.</t>
         </is>
       </c>
       <c r="H4" s="2" t="str">

</xml_diff>